<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-08-20
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3382,7 +3382,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Por</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -4155,7 +4155,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -4268,7 +4268,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E;W</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5107,7 +5107,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5335,7 +5335,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5449,7 +5449,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5506,7 +5506,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5734,7 +5734,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5857,7 +5857,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5996,7 +5996,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -6053,7 +6053,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Dd;E</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Dd;E</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -6281,7 +6281,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -6338,7 +6338,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -6509,7 +6509,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -6566,7 +6566,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -6680,7 +6680,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Dd;E</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -6794,7 +6794,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -6851,7 +6851,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -6965,7 +6965,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -7022,7 +7022,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -7193,7 +7193,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -7535,7 +7535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -7592,7 +7592,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -7649,7 +7649,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -7763,7 +7763,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -7991,7 +7991,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -8048,7 +8048,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -8105,7 +8105,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -8162,7 +8162,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -8219,7 +8219,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -8383,7 +8383,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -8424,7 +8424,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -8506,7 +8506,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -8661,7 +8661,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -8832,7 +8832,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -8889,7 +8889,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Dd;E</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -8946,7 +8946,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -9060,7 +9060,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -9117,7 +9117,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -9231,7 +9231,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;Dc</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -9288,7 +9288,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -9459,7 +9459,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -9573,7 +9573,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -9630,7 +9630,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -9687,7 +9687,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -9801,7 +9801,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -9915,7 +9915,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -10200,7 +10200,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -10257,7 +10257,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -10371,7 +10371,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -10485,7 +10485,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -10542,7 +10542,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -10599,7 +10599,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -10681,7 +10681,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -10722,7 +10722,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -10763,7 +10763,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -10804,7 +10804,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -10845,7 +10845,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -10927,7 +10927,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -10968,7 +10968,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -11009,7 +11009,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -11132,7 +11132,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -11173,7 +11173,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -11255,7 +11255,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -11296,7 +11296,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -11353,7 +11353,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -11410,7 +11410,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -11467,7 +11467,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -11524,7 +11524,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -11581,7 +11581,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -11638,7 +11638,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -11695,7 +11695,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -11752,7 +11752,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -11809,7 +11809,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -11866,7 +11866,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -11980,7 +11980,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -12037,7 +12037,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -12094,7 +12094,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -12151,7 +12151,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -12265,7 +12265,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -12322,7 +12322,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -12379,7 +12379,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -12436,7 +12436,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -12534,7 +12534,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -12616,7 +12616,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -12657,7 +12657,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -12698,7 +12698,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -12739,7 +12739,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -12780,7 +12780,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -12862,7 +12862,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -12985,7 +12985,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -13026,7 +13026,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -13067,7 +13067,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -13108,7 +13108,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -13165,7 +13165,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -13222,7 +13222,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -13336,7 +13336,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -13418,7 +13418,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -13459,7 +13459,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -13662,7 +13662,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T;A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -13719,7 +13719,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -13833,7 +13833,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T;A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -13947,7 +13947,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T;A</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -14004,7 +14004,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -14061,7 +14061,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -14118,7 +14118,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -14159,7 +14159,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -14216,7 +14216,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -14330,7 +14330,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -14501,7 +14501,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -14558,7 +14558,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -14729,7 +14729,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -14786,7 +14786,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -14843,7 +14843,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -14957,7 +14957,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T;A</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -15014,7 +15014,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E;W</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -15071,7 +15071,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -15185,7 +15185,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -15242,7 +15242,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -15413,7 +15413,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -15470,7 +15470,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -15527,7 +15527,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -15609,7 +15609,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -15707,7 +15707,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -15821,7 +15821,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -15935,7 +15935,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -15992,7 +15992,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -16106,7 +16106,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -16220,7 +16220,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -16277,7 +16277,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -16334,7 +16334,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -16391,7 +16391,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -16448,7 +16448,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -16505,7 +16505,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -16562,7 +16562,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -16619,7 +16619,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -16676,7 +16676,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -16733,7 +16733,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -16790,7 +16790,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -16904,7 +16904,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -16961,7 +16961,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -17075,7 +17075,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -17132,7 +17132,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E;C</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -17189,7 +17189,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -17246,7 +17246,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E;C</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -17303,7 +17303,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -17417,7 +17417,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -17474,7 +17474,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -17531,7 +17531,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -17588,7 +17588,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -17645,7 +17645,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -17702,7 +17702,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -17759,7 +17759,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -17816,7 +17816,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -17873,7 +17873,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -17914,7 +17914,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -17955,7 +17955,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -17996,7 +17996,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -18037,7 +18037,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -18078,7 +18078,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E;W</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -18119,7 +18119,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -18233,7 +18233,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -18290,7 +18290,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -18347,7 +18347,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -18404,7 +18404,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -18461,7 +18461,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -18518,7 +18518,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -18575,7 +18575,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -18632,7 +18632,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -18689,7 +18689,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -18746,7 +18746,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -18803,7 +18803,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -18860,7 +18860,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -18917,7 +18917,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E;W</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -18974,7 +18974,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -19031,7 +19031,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -19088,7 +19088,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -19145,7 +19145,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -19202,7 +19202,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -19316,7 +19316,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -19373,7 +19373,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -19430,7 +19430,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -19487,7 +19487,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -19544,7 +19544,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -19601,7 +19601,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E;M</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -19658,7 +19658,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -19715,7 +19715,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -19772,7 +19772,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -20000,7 +20000,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -20057,7 +20057,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -20114,7 +20114,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -20171,7 +20171,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -20228,7 +20228,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -20342,7 +20342,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -20383,7 +20383,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -20424,7 +20424,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -20465,7 +20465,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -20506,7 +20506,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -20547,7 +20547,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -20588,7 +20588,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -20629,7 +20629,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -20670,7 +20670,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -20711,7 +20711,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -20752,7 +20752,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -20793,7 +20793,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -20875,7 +20875,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -20916,7 +20916,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -20957,7 +20957,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -21014,7 +21014,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -21071,7 +21071,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -21128,7 +21128,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -21185,7 +21185,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -21242,7 +21242,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -21299,7 +21299,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;W</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -21356,7 +21356,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -21413,7 +21413,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -21470,7 +21470,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -21527,7 +21527,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -21584,7 +21584,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -21641,7 +21641,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -21698,7 +21698,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -21755,7 +21755,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -21812,7 +21812,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -21926,7 +21926,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -21983,7 +21983,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -22040,7 +22040,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -22097,7 +22097,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -22154,7 +22154,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -22211,7 +22211,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -22268,7 +22268,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -22325,7 +22325,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -22382,7 +22382,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -22439,7 +22439,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -22496,7 +22496,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -22537,7 +22537,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -22578,7 +22578,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -22619,7 +22619,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -22660,7 +22660,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E;W</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -22701,7 +22701,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -22783,7 +22783,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -22865,7 +22865,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -22922,7 +22922,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E;C</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -22979,7 +22979,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -23036,7 +23036,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -23093,7 +23093,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -23150,7 +23150,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -23207,7 +23207,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -23289,7 +23289,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -23451,7 +23451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -23508,7 +23508,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -23565,7 +23565,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -23622,7 +23622,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -23679,7 +23679,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -23777,7 +23777,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -23834,7 +23834,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -23891,7 +23891,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -24005,7 +24005,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -24119,7 +24119,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -24176,7 +24176,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -24290,7 +24290,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -24347,7 +24347,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -24461,7 +24461,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -24616,7 +24616,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -24730,7 +24730,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -24787,7 +24787,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -24844,7 +24844,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -24901,7 +24901,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -25072,7 +25072,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -25129,7 +25129,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -25186,7 +25186,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -25243,7 +25243,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -25357,7 +25357,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -25414,7 +25414,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -25471,7 +25471,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -25528,7 +25528,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -25569,7 +25569,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -25610,7 +25610,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -25651,7 +25651,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -25790,7 +25790,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -25847,7 +25847,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -25961,7 +25961,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -26132,7 +26132,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -26189,7 +26189,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -26246,7 +26246,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -26303,7 +26303,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>T;A</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -26531,7 +26531,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -26588,7 +26588,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -26645,7 +26645,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -26702,7 +26702,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -26816,7 +26816,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -26857,7 +26857,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -26898,7 +26898,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -26939,7 +26939,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -27021,7 +27021,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -27062,7 +27062,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -27144,7 +27144,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -27201,7 +27201,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -27258,7 +27258,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -27315,7 +27315,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -27372,7 +27372,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -27429,7 +27429,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -27486,7 +27486,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -27543,7 +27543,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -27600,7 +27600,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -27657,7 +27657,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -27771,7 +27771,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -27828,7 +27828,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -27885,7 +27885,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -27926,7 +27926,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -28008,7 +28008,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -28065,7 +28065,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -28106,7 +28106,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -28147,7 +28147,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-08-21
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Portieri'!$A$1:$S$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Difensori'!$A$1:$Q$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Difensori'!$A$1:$Q$177</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Centrocampisti'!$A$1:$Q$181</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Attaccanti'!$A$1:$Q$90</definedName>
   </definedNames>
@@ -4151,7 +4151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q178"/>
+  <dimension ref="A1:Q177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12980,27 +12980,27 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Matturro</t>
+          <t>Bakoune</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Ds;Dc</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D167" t="n">
         <v>1</v>
       </c>
       <c r="E167" t="n">
+        <v>4</v>
+      </c>
+      <c r="F167" t="n">
         <v>2</v>
-      </c>
-      <c r="F167" t="n">
-        <v>1</v>
       </c>
       <c r="G167" s="6" t="inlineStr">
         <is>
@@ -13021,24 +13021,24 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Bakoune</t>
+          <t>Abankwah</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="D168" t="n">
         <v>1</v>
       </c>
       <c r="E168" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F168" t="n">
         <v>2</v>
@@ -13062,40 +13062,56 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Abankwah</t>
+          <t>Ziolkowski</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Dd;Dc</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="D169" t="n">
         <v>1</v>
       </c>
       <c r="E169" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F169" t="n">
-        <v>2</v>
-      </c>
-      <c r="G169" s="6" t="inlineStr">
-        <is>
-          <t>Low Cost</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr"/>
-      <c r="I169" t="inlineStr"/>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
-      <c r="M169" t="inlineStr"/>
-      <c r="N169" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G169" s="7" t="inlineStr">
+        <is>
+          <t>Scommessa</t>
+        </is>
+      </c>
+      <c r="H169" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Affare</t>
+        </is>
+      </c>
+      <c r="J169" t="n">
+        <v>9</v>
+      </c>
+      <c r="K169" t="n">
+        <v>5.94</v>
+      </c>
+      <c r="L169" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="M169" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
       <c r="O169" t="inlineStr"/>
       <c r="P169" t="inlineStr"/>
       <c r="Q169" t="inlineStr"/>
@@ -13103,7 +13119,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Ziolkowski</t>
+          <t>Goldaniga</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -13113,17 +13129,17 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D170" t="n">
         <v>1</v>
       </c>
       <c r="E170" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F170" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G170" s="7" t="inlineStr">
         <is>
@@ -13131,21 +13147,21 @@
         </is>
       </c>
       <c r="H170" t="n">
-        <v>23.6</v>
+        <v>12.6</v>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Affare</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J170" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K170" t="n">
-        <v>5.94</v>
+        <v>0</v>
       </c>
       <c r="L170" t="n">
-        <v>5.78</v>
+        <v>0</v>
       </c>
       <c r="M170" t="n">
         <v>0</v>
@@ -13160,27 +13176,27 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Goldaniga</t>
+          <t>Missori</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D171" t="n">
         <v>1</v>
       </c>
       <c r="E171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G171" s="7" t="inlineStr">
         <is>
@@ -13217,12 +13233,12 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Missori</t>
+          <t>Pieragnolo</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -13234,10 +13250,10 @@
         <v>1</v>
       </c>
       <c r="E172" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G172" s="7" t="inlineStr">
         <is>
@@ -13274,17 +13290,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Pieragnolo</t>
+          <t>Amey</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -13301,29 +13317,13 @@
           <t>Scommessa</t>
         </is>
       </c>
-      <c r="H173" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J173" t="n">
-        <v>0</v>
-      </c>
-      <c r="K173" t="n">
-        <v>0</v>
-      </c>
-      <c r="L173" t="n">
-        <v>0</v>
-      </c>
-      <c r="M173" t="n">
-        <v>0</v>
-      </c>
-      <c r="N173" t="n">
-        <v>0</v>
-      </c>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr"/>
+      <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr"/>
       <c r="P173" t="inlineStr"/>
       <c r="Q173" t="inlineStr"/>
@@ -13331,27 +13331,27 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Amey</t>
+          <t>Matturro</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D174" t="n">
         <v>1</v>
       </c>
       <c r="E174" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G174" s="7" t="inlineStr">
         <is>
@@ -13372,7 +13372,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Gelli J.</t>
+          <t>Antov</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -13382,17 +13382,17 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D175" t="n">
         <v>1</v>
       </c>
       <c r="E175" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F175" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G175" s="7" t="inlineStr">
         <is>
@@ -13413,27 +13413,27 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Antov</t>
+          <t>Gomes</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D176" t="n">
         <v>1</v>
       </c>
       <c r="E176" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F176" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G176" s="7" t="inlineStr">
         <is>
@@ -13454,17 +13454,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Gomes</t>
+          <t>Omar Fayed</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Ds;Dc</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -13492,49 +13492,8 @@
       <c r="P177" t="inlineStr"/>
       <c r="Q177" t="inlineStr"/>
     </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>Omar Fayed</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>Dc</t>
-        </is>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>Frosinone</t>
-        </is>
-      </c>
-      <c r="D178" t="n">
-        <v>1</v>
-      </c>
-      <c r="E178" t="n">
-        <v>1</v>
-      </c>
-      <c r="F178" t="n">
-        <v>0</v>
-      </c>
-      <c r="G178" s="7" t="inlineStr">
-        <is>
-          <t>Scommessa</t>
-        </is>
-      </c>
-      <c r="H178" t="inlineStr"/>
-      <c r="I178" t="inlineStr"/>
-      <c r="J178" t="inlineStr"/>
-      <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
-      <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
-      <c r="O178" t="inlineStr"/>
-      <c r="P178" t="inlineStr"/>
-      <c r="Q178" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q178"/>
+  <autoFilter ref="A1:Q177"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-08-25
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Portieri'!$A$1:$AA$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Difensori'!$A$1:$AA$184</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Centrocampisti'!$A$1:$AA$184</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Attaccanti'!$A$1:$AA$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Attaccanti'!$A$1:$AA$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -1287,10 +1287,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -6087,10 +6087,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -6172,10 +6172,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -7536,10 +7536,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -7708,10 +7708,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -8400,10 +8400,10 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T30" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -9623,10 +9623,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U45" t="n">
         <v>0</v>
@@ -12197,10 +12197,10 @@
       <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T75" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U75" t="n">
         <v>0</v>
@@ -13723,10 +13723,10 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T95" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U95" t="n">
         <v>0</v>
@@ -13810,10 +13810,10 @@
         <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T96" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U96" t="n">
         <v>0</v>
@@ -21752,10 +21752,10 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T10" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -22962,10 +22962,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U24" t="n">
         <v>0</v>
@@ -23308,10 +23308,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T28" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U28" t="n">
         <v>0</v>
@@ -23865,10 +23865,10 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T35" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
@@ -24157,10 +24157,10 @@
         <v>1</v>
       </c>
       <c r="S39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T39" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U39" t="n">
         <v>0</v>
@@ -25282,10 +25282,10 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T52" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="U52" t="n">
         <v>0</v>
@@ -26063,10 +26063,10 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T61" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U61" t="n">
         <v>0</v>
@@ -27018,10 +27018,10 @@
         <v>0</v>
       </c>
       <c r="S72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T72" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U72" t="n">
         <v>0</v>
@@ -27636,10 +27636,10 @@
       <c r="Q80" t="inlineStr"/>
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T80" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U80" t="n">
         <v>0</v>
@@ -28250,10 +28250,10 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T88" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U88" t="n">
         <v>0</v>
@@ -28337,13 +28337,13 @@
         <v>0</v>
       </c>
       <c r="S89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T89" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="U89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V89" t="n">
         <v>0</v>
@@ -36161,7 +36161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA87"/>
+  <dimension ref="A1:AA88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -36653,13 +36653,13 @@
         <v>4</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5" t="n">
-        <v>0</v>
+        <v>17.5</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V5" t="n">
         <v>0</v>
@@ -37408,10 +37408,10 @@
         <v>2</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -37667,16 +37667,16 @@
         <v>1</v>
       </c>
       <c r="S17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T17" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W17" t="n">
         <v>0</v>
@@ -37778,7 +37778,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Simeone</t>
+          <t>Castro S.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -37788,17 +37788,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E19" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F19" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
@@ -37806,36 +37806,36 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>59.5</v>
+        <v>61.1</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Trappola</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K19" t="n">
-        <v>6.08</v>
+        <v>5.93</v>
       </c>
       <c r="L19" t="n">
-        <v>7.09</v>
+        <v>6.51</v>
       </c>
       <c r="M19" t="n">
         <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>1.09</v>
+        <v>-0.15</v>
       </c>
       <c r="O19" t="n">
-        <v>0.596</v>
+        <v>0.64</v>
       </c>
       <c r="P19" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
@@ -37844,7 +37844,7 @@
         <v>1</v>
       </c>
       <c r="T19" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -37853,7 +37853,7 @@
         <v>0</v>
       </c>
       <c r="W19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X19" t="n">
         <v>0</v>
@@ -37865,73 +37865,73 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Leao</t>
+          <t>Simeone</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E20" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F20" t="n">
-        <v>38</v>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>2a Fascia</t>
+        <v>40</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>1a Fascia</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>84.5</v>
+        <v>59.5</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Trappola</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="K20" t="n">
-        <v>5.88</v>
+        <v>6.08</v>
       </c>
       <c r="L20" t="n">
-        <v>6.86</v>
+        <v>7.09</v>
       </c>
       <c r="M20" t="n">
         <v>3</v>
       </c>
       <c r="N20" t="n">
-        <v>-0.33</v>
+        <v>1.09</v>
       </c>
       <c r="O20" t="n">
-        <v>0.833</v>
+        <v>0.596</v>
       </c>
       <c r="P20" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -37940,7 +37940,7 @@
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="X20" t="n">
         <v>0</v>
@@ -37952,7 +37952,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Esposito Se.</t>
+          <t>Leao</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -37962,17 +37962,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E21" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="F21" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -37980,39 +37980,39 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>77.40000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Affare</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="K21" t="n">
-        <v>6.26</v>
+        <v>5.88</v>
       </c>
       <c r="L21" t="n">
-        <v>6.88</v>
+        <v>6.86</v>
       </c>
       <c r="M21" t="n">
         <v>3</v>
       </c>
       <c r="N21" t="n">
-        <v>2.64</v>
+        <v>-0.33</v>
       </c>
       <c r="O21" t="n">
-        <v>0.605</v>
+        <v>0.833</v>
       </c>
       <c r="P21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S21" t="n">
         <v>0</v>
@@ -38027,7 +38027,7 @@
         <v>0</v>
       </c>
       <c r="W21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X21" t="n">
         <v>0</v>
@@ -38039,7 +38039,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Soulè</t>
+          <t>Esposito Se.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -38049,17 +38049,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E22" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F22" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
@@ -38067,54 +38067,54 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>76.7</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Affare</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="K22" t="n">
-        <v>6.12</v>
+        <v>6.26</v>
       </c>
       <c r="L22" t="n">
-        <v>6.83</v>
+        <v>6.88</v>
       </c>
       <c r="M22" t="n">
         <v>3</v>
       </c>
       <c r="N22" t="n">
-        <v>-0.22</v>
+        <v>2.64</v>
       </c>
       <c r="O22" t="n">
-        <v>0.798</v>
+        <v>0.605</v>
       </c>
       <c r="P22" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>4</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="n">
         <v>6</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>5</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" t="n">
-        <v>0</v>
-      </c>
-      <c r="T22" t="n">
-        <v>0</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" t="n">
-        <v>0</v>
-      </c>
-      <c r="W22" t="n">
-        <v>1</v>
       </c>
       <c r="X22" t="n">
         <v>0</v>
@@ -38126,27 +38126,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pinamonti</t>
+          <t>Soulè</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E23" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F23" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -38154,7 +38154,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>74.2</v>
+        <v>76.7</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -38162,37 +38162,37 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K23" t="n">
-        <v>5.88</v>
+        <v>6.12</v>
       </c>
       <c r="L23" t="n">
-        <v>6.62</v>
+        <v>6.83</v>
       </c>
       <c r="M23" t="n">
         <v>3</v>
       </c>
       <c r="N23" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.22</v>
       </c>
       <c r="O23" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.798</v>
       </c>
       <c r="P23" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Q23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -38201,10 +38201,10 @@
         <v>0</v>
       </c>
       <c r="W23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
@@ -38213,85 +38213,85 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Adams C.</t>
+          <t>Pinamonti</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D24" t="n">
+        <v>13</v>
+      </c>
+      <c r="E24" t="n">
+        <v>51</v>
+      </c>
+      <c r="F24" t="n">
+        <v>26</v>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>2a Fascia</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>34</v>
+      </c>
+      <c r="K24" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="L24" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="M24" t="n">
+        <v>3</v>
+      </c>
+      <c r="N24" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="P24" t="n">
         <v>9</v>
-      </c>
-      <c r="E24" t="n">
-        <v>33</v>
-      </c>
-      <c r="F24" t="n">
-        <v>16</v>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>2a Fascia</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>71.5</v>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Affare</t>
-        </is>
-      </c>
-      <c r="J24" t="n">
-        <v>32</v>
-      </c>
-      <c r="K24" t="n">
-        <v>5.98</v>
-      </c>
-      <c r="L24" t="n">
-        <v>6.64</v>
-      </c>
-      <c r="M24" t="n">
-        <v>2</v>
-      </c>
-      <c r="N24" t="n">
-        <v>-0.12</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.882</v>
-      </c>
-      <c r="P24" t="n">
-        <v>6</v>
       </c>
       <c r="Q24" t="n">
         <v>3</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T24" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
@@ -38300,65 +38300,65 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dovbyk</t>
+          <t>Adams C.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D25" t="n">
+        <v>9</v>
+      </c>
+      <c r="E25" t="n">
+        <v>33</v>
+      </c>
+      <c r="F25" t="n">
         <v>16</v>
       </c>
-      <c r="E25" t="n">
-        <v>58</v>
-      </c>
-      <c r="F25" t="n">
-        <v>29</v>
-      </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
           <t>2a Fascia</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>63.6</v>
+        <v>71.5</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Affare</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="K25" t="n">
-        <v>6</v>
+        <v>5.98</v>
       </c>
       <c r="L25" t="n">
-        <v>6.77</v>
+        <v>6.64</v>
       </c>
       <c r="M25" t="n">
         <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>-0.42</v>
+        <v>-0.12</v>
       </c>
       <c r="O25" t="n">
-        <v>0.592</v>
+        <v>0.882</v>
       </c>
       <c r="P25" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q25" t="n">
         <v>3</v>
       </c>
-      <c r="Q25" t="n">
-        <v>1</v>
-      </c>
       <c r="R25" t="n">
         <v>0</v>
       </c>
@@ -38366,10 +38366,10 @@
         <v>1</v>
       </c>
       <c r="T25" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V25" t="n">
         <v>0</v>
@@ -38387,7 +38387,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Castro S.</t>
+          <t>Dovbyk</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -38397,17 +38397,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E26" t="n">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="F26" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
@@ -38415,7 +38415,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>61.1</v>
+        <v>63.6</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -38423,26 +38423,26 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="K26" t="n">
-        <v>5.93</v>
+        <v>6</v>
       </c>
       <c r="L26" t="n">
-        <v>6.51</v>
+        <v>6.77</v>
       </c>
       <c r="M26" t="n">
+        <v>2</v>
+      </c>
+      <c r="N26" t="n">
+        <v>-0.42</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.592</v>
+      </c>
+      <c r="P26" t="n">
         <v>3</v>
       </c>
-      <c r="N26" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="P26" t="n">
-        <v>7</v>
-      </c>
       <c r="Q26" t="n">
         <v>1</v>
       </c>
@@ -38450,10 +38450,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -38462,7 +38462,7 @@
         <v>0</v>
       </c>
       <c r="W26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X26" t="n">
         <v>0</v>
@@ -38537,10 +38537,10 @@
         <v>1</v>
       </c>
       <c r="S27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T27" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -39338,27 +39338,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Yeboah J.</t>
+          <t>Tourè E.</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E37" t="n">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="F37" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
@@ -39366,7 +39366,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>33.6</v>
+        <v>33.2</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -39374,26 +39374,28 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>5.91</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>5.98</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
-      </c>
-      <c r="N37" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N37" t="n">
+        <v>-2.46</v>
+      </c>
       <c r="O37" t="n">
-        <v>0.737</v>
+        <v>0.079</v>
       </c>
       <c r="P37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -39402,7 +39404,7 @@
         <v>1</v>
       </c>
       <c r="T37" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -39411,7 +39413,7 @@
         <v>0</v>
       </c>
       <c r="W37" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X37" t="n">
         <v>0</v>
@@ -39423,27 +39425,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Tourè E.</t>
+          <t>Ghedjemis</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E38" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="F38" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
@@ -39451,7 +39453,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>33.2</v>
+        <v>13.6</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -39459,22 +39461,20 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>6.1</v>
       </c>
       <c r="M38" t="n">
-        <v>3</v>
-      </c>
-      <c r="N38" t="n">
-        <v>-2.46</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" t="n">
-        <v>0.079</v>
+        <v>0.132</v>
       </c>
       <c r="P38" t="n">
         <v>0</v>
@@ -39486,10 +39486,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T38" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -39498,7 +39498,7 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X38" t="n">
         <v>0</v>
@@ -39510,66 +39510,46 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ghedjemis</t>
+          <t>Kevin Carlos</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>W;A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E39" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="F39" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
           <t>2a Fascia</t>
         </is>
       </c>
-      <c r="H39" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Trappola</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>5</v>
-      </c>
-      <c r="K39" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="L39" t="n">
-        <v>6.1</v>
-      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="P39" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" t="n">
-        <v>0</v>
-      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
       <c r="S39" t="n">
         <v>0</v>
       </c>
@@ -39582,12 +39562,8 @@
       <c r="V39" t="n">
         <v>0</v>
       </c>
-      <c r="W39" t="n">
-        <v>1</v>
-      </c>
-      <c r="X39" t="n">
-        <v>0</v>
-      </c>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr"/>
@@ -39595,7 +39571,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kevin Carlos</t>
+          <t>Adams A.</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -39605,17 +39581,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E40" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="F40" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
@@ -39636,10 +39612,10 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T40" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U40" t="n">
         <v>0</v>
@@ -39656,7 +39632,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Adams A.</t>
+          <t>Romero D.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -39666,17 +39642,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E41" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="F41" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
@@ -39697,10 +39673,10 @@
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="U41" t="n">
         <v>0</v>
@@ -39717,7 +39693,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Romero D.</t>
+          <t>Osmajic</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -39727,17 +39703,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E42" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F42" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
@@ -40984,7 +40960,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Lang</t>
+          <t>Yeboah J.</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -40994,17 +40970,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E57" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F57" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
@@ -41012,28 +40988,28 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>32.2</v>
+        <v>33.6</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Trappola</t>
         </is>
       </c>
       <c r="J57" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="K57" t="n">
-        <v>6.04</v>
+        <v>5.91</v>
       </c>
       <c r="L57" t="n">
-        <v>6.32</v>
+        <v>5.98</v>
       </c>
       <c r="M57" t="n">
         <v>1</v>
       </c>
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
-        <v>0.368</v>
+        <v>0.737</v>
       </c>
       <c r="P57" t="n">
         <v>1</v>
@@ -41057,7 +41033,7 @@
         <v>0</v>
       </c>
       <c r="W57" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="X57" t="n">
         <v>0</v>
@@ -41069,35 +41045,35 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Gimenez</t>
+          <t>Lang</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D58" t="n">
+        <v>3</v>
+      </c>
+      <c r="E58" t="n">
+        <v>12</v>
+      </c>
+      <c r="F58" t="n">
         <v>6</v>
       </c>
-      <c r="E58" t="n">
-        <v>10</v>
-      </c>
-      <c r="F58" t="n">
-        <v>5</v>
-      </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
           <t>3a Fascia</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>25.3</v>
+        <v>32.2</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -41105,37 +41081,35 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K58" t="n">
-        <v>5.5</v>
+        <v>6.04</v>
       </c>
       <c r="L58" t="n">
-        <v>5.53</v>
+        <v>6.32</v>
       </c>
       <c r="M58" t="n">
+        <v>1</v>
+      </c>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="n">
+        <v>0.368</v>
+      </c>
+      <c r="P58" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q58" t="n">
         <v>2</v>
       </c>
-      <c r="N58" t="n">
-        <v>-1.22</v>
-      </c>
-      <c r="O58" t="n">
-        <v>0.355</v>
-      </c>
-      <c r="P58" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q58" t="n">
-        <v>1</v>
-      </c>
       <c r="R58" t="n">
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T58" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U58" t="n">
         <v>0</v>
@@ -41156,82 +41130,82 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>N'Dri</t>
+          <t>Gimenez</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>W;A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E59" t="n">
+        <v>10</v>
+      </c>
+      <c r="F59" t="n">
+        <v>5</v>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>3a Fascia</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
         <v>15</v>
       </c>
-      <c r="F59" t="n">
-        <v>8</v>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>3a Fascia</t>
-        </is>
-      </c>
-      <c r="H59" t="n">
-        <v>21.9</v>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J59" t="n">
-        <v>17</v>
-      </c>
       <c r="K59" t="n">
-        <v>5.82</v>
+        <v>5.5</v>
       </c>
       <c r="L59" t="n">
-        <v>6.09</v>
+        <v>5.53</v>
       </c>
       <c r="M59" t="n">
         <v>2</v>
       </c>
       <c r="N59" t="n">
-        <v>0.23</v>
+        <v>-1.22</v>
       </c>
       <c r="O59" t="n">
-        <v>0.316</v>
+        <v>0.355</v>
       </c>
       <c r="P59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>1</v>
+      </c>
+      <c r="R59" t="n">
+        <v>0</v>
+      </c>
+      <c r="S59" t="n">
+        <v>0</v>
+      </c>
+      <c r="T59" t="n">
+        <v>0</v>
+      </c>
+      <c r="U59" t="n">
+        <v>0</v>
+      </c>
+      <c r="V59" t="n">
+        <v>0</v>
+      </c>
+      <c r="W59" t="n">
         <v>2</v>
-      </c>
-      <c r="Q59" t="n">
-        <v>0</v>
-      </c>
-      <c r="R59" t="n">
-        <v>0</v>
-      </c>
-      <c r="S59" t="n">
-        <v>1</v>
-      </c>
-      <c r="T59" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="U59" t="n">
-        <v>0</v>
-      </c>
-      <c r="V59" t="n">
-        <v>0</v>
-      </c>
-      <c r="W59" t="n">
-        <v>3</v>
       </c>
       <c r="X59" t="n">
         <v>0</v>
@@ -41243,27 +41217,27 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Camarda</t>
+          <t>N'Dri</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E60" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F60" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
@@ -41271,54 +41245,54 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>15</v>
+        <v>21.9</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Trappola</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J60" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K60" t="n">
-        <v>5.67</v>
+        <v>5.82</v>
       </c>
       <c r="L60" t="n">
-        <v>5.64</v>
+        <v>6.09</v>
       </c>
       <c r="M60" t="n">
+        <v>2</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0.316</v>
+      </c>
+      <c r="P60" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>0</v>
+      </c>
+      <c r="R60" t="n">
+        <v>0</v>
+      </c>
+      <c r="S60" t="n">
+        <v>1</v>
+      </c>
+      <c r="T60" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="U60" t="n">
+        <v>0</v>
+      </c>
+      <c r="V60" t="n">
+        <v>0</v>
+      </c>
+      <c r="W60" t="n">
         <v>3</v>
-      </c>
-      <c r="N60" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="O60" t="n">
-        <v>0.211</v>
-      </c>
-      <c r="P60" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q60" t="n">
-        <v>0</v>
-      </c>
-      <c r="R60" t="n">
-        <v>1</v>
-      </c>
-      <c r="S60" t="n">
-        <v>0</v>
-      </c>
-      <c r="T60" t="n">
-        <v>0</v>
-      </c>
-      <c r="U60" t="n">
-        <v>0</v>
-      </c>
-      <c r="V60" t="n">
-        <v>0</v>
-      </c>
-      <c r="W60" t="n">
-        <v>1</v>
       </c>
       <c r="X60" t="n">
         <v>0</v>
@@ -41330,7 +41304,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Mutandwa</t>
+          <t>Camarda</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -41340,55 +41314,57 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E61" t="n">
+        <v>20</v>
+      </c>
+      <c r="F61" t="n">
         <v>10</v>
       </c>
-      <c r="F61" t="n">
-        <v>5</v>
-      </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
           <t>3a Fascia</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Trappola</t>
         </is>
       </c>
       <c r="J61" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="K61" t="n">
-        <v>5.9</v>
+        <v>5.67</v>
       </c>
       <c r="L61" t="n">
-        <v>5.9</v>
+        <v>5.64</v>
       </c>
       <c r="M61" t="n">
-        <v>1</v>
-      </c>
-      <c r="N61" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N61" t="n">
+        <v>1.94</v>
+      </c>
       <c r="O61" t="n">
-        <v>0.132</v>
+        <v>0.211</v>
       </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q61" t="n">
         <v>0</v>
       </c>
       <c r="R61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S61" t="n">
         <v>0</v>
@@ -41403,7 +41379,7 @@
         <v>0</v>
       </c>
       <c r="W61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X61" t="n">
         <v>0</v>
@@ -41415,27 +41391,27 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Kvernadze</t>
+          <t>Mutandwa</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>W;A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E62" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F62" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
@@ -41443,28 +41419,28 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Trappola</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K62" t="n">
-        <v>5.75</v>
+        <v>5.9</v>
       </c>
       <c r="L62" t="n">
-        <v>5.75</v>
+        <v>5.9</v>
       </c>
       <c r="M62" t="n">
         <v>1</v>
       </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="n">
-        <v>0.053</v>
+        <v>0.132</v>
       </c>
       <c r="P62" t="n">
         <v>0</v>
@@ -41476,10 +41452,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U62" t="n">
         <v>0</v>
@@ -41500,27 +41476,27 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Ratkov</t>
+          <t>Kvernadze</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E63" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F63" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
@@ -41528,7 +41504,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>8.6</v>
+        <v>9.5</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -41536,20 +41512,20 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>5.64</v>
+        <v>5.75</v>
       </c>
       <c r="L63" t="n">
-        <v>5.64</v>
+        <v>5.75</v>
       </c>
       <c r="M63" t="n">
         <v>1</v>
       </c>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="n">
-        <v>0.184</v>
+        <v>0.053</v>
       </c>
       <c r="P63" t="n">
         <v>0</v>
@@ -41561,10 +41537,10 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T63" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U63" t="n">
         <v>0</v>
@@ -41585,7 +41561,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Raimondo</t>
+          <t>Ratkov</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -41595,48 +41571,46 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D64" t="n">
+        <v>10</v>
+      </c>
+      <c r="E64" t="n">
+        <v>26</v>
+      </c>
+      <c r="F64" t="n">
+        <v>13</v>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>3a Fascia</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Trappola</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
         <v>7</v>
       </c>
-      <c r="E64" t="n">
-        <v>22</v>
-      </c>
-      <c r="F64" t="n">
-        <v>11</v>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
-        <is>
-          <t>3a Fascia</t>
-        </is>
-      </c>
-      <c r="H64" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Trappola</t>
-        </is>
-      </c>
-      <c r="J64" t="n">
-        <v>1</v>
-      </c>
       <c r="K64" t="n">
-        <v>6</v>
+        <v>5.64</v>
       </c>
       <c r="L64" t="n">
-        <v>6</v>
+        <v>5.64</v>
       </c>
       <c r="M64" t="n">
-        <v>2</v>
-      </c>
-      <c r="N64" t="n">
-        <v>6</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N64" t="inlineStr"/>
       <c r="O64" t="n">
-        <v>0.013</v>
+        <v>0.184</v>
       </c>
       <c r="P64" t="n">
         <v>0</v>
@@ -41648,10 +41622,10 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="U64" t="n">
         <v>0</v>
@@ -41672,27 +41646,27 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Frigan</t>
+          <t>Raimondo</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E65" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F65" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
@@ -41700,28 +41674,30 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>5.8</v>
+        <v>6.9</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Trappola</t>
         </is>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K65" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L65" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M65" t="n">
-        <v>1</v>
-      </c>
-      <c r="N65" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="N65" t="n">
+        <v>6</v>
+      </c>
       <c r="O65" t="n">
-        <v>0</v>
+        <v>0.013</v>
       </c>
       <c r="P65" t="n">
         <v>0</v>
@@ -41733,10 +41709,10 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T65" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
@@ -42883,46 +42859,66 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Havel</t>
+          <t>Frigan</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E80" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
           <t>Low Cost</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
+      <c r="H80" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
       <c r="M80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
-      <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
+      <c r="O80" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0</v>
+      </c>
       <c r="S80" t="n">
         <v>0</v>
       </c>
@@ -42935,8 +42931,12 @@
       <c r="V80" t="n">
         <v>0</v>
       </c>
-      <c r="W80" t="inlineStr"/>
-      <c r="X80" t="inlineStr"/>
+      <c r="W80" t="n">
+        <v>0</v>
+      </c>
+      <c r="X80" t="n">
+        <v>0</v>
+      </c>
       <c r="Y80" t="inlineStr"/>
       <c r="Z80" t="inlineStr"/>
       <c r="AA80" t="inlineStr"/>
@@ -42944,27 +42944,27 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Robinson J.</t>
+          <t>Havel</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>4</v>
       </c>
       <c r="E81" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G81" s="6" t="inlineStr">
         <is>
@@ -43005,12 +43005,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Varela G.</t>
+          <t>Robinson J.</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -43019,13 +43019,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E82" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F82" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
@@ -43046,13 +43046,13 @@
       <c r="Q82" t="inlineStr"/>
       <c r="R82" t="inlineStr"/>
       <c r="S82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T82" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U82" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V82" t="n">
         <v>0</v>
@@ -43066,27 +43066,27 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Lontani</t>
+          <t>Varela G.</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E83" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G83" s="6" t="inlineStr">
         <is>
@@ -43110,10 +43110,10 @@
         <v>1</v>
       </c>
       <c r="T83" t="n">
-        <v>6.5</v>
+        <v>10</v>
       </c>
       <c r="U83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V83" t="n">
         <v>0</v>
@@ -43127,73 +43127,51 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Azon</t>
+          <t>Lontani</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D84" t="n">
         <v>1</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F84" t="n">
-        <v>1</v>
-      </c>
-      <c r="G84" s="7" t="inlineStr">
-        <is>
-          <t>Scommessa</t>
-        </is>
-      </c>
-      <c r="H84" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J84" t="n">
-        <v>0</v>
-      </c>
-      <c r="K84" t="n">
-        <v>0</v>
-      </c>
-      <c r="L84" t="n">
-        <v>0</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>Low Cost</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
       <c r="M84" t="n">
-        <v>2</v>
-      </c>
-      <c r="N84" t="n">
-        <v>0</v>
-      </c>
-      <c r="O84" t="n">
-        <v>0</v>
-      </c>
-      <c r="P84" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q84" t="n">
-        <v>0</v>
-      </c>
-      <c r="R84" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T84" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="U84" t="n">
         <v>0</v>
@@ -43201,12 +43179,8 @@
       <c r="V84" t="n">
         <v>0</v>
       </c>
-      <c r="W84" t="n">
-        <v>0</v>
-      </c>
-      <c r="X84" t="n">
-        <v>0</v>
-      </c>
+      <c r="W84" t="inlineStr"/>
+      <c r="X84" t="inlineStr"/>
       <c r="Y84" t="inlineStr"/>
       <c r="Z84" t="inlineStr"/>
       <c r="AA84" t="inlineStr"/>
@@ -43214,17 +43188,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Lisman</t>
+          <t>Azon</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>W;A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -43241,19 +43215,41 @@
           <t>Scommessa</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
+      <c r="H85" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
       <c r="M85" t="n">
-        <v>0</v>
-      </c>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
-      <c r="P85" t="inlineStr"/>
-      <c r="Q85" t="inlineStr"/>
-      <c r="R85" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>0</v>
+      </c>
+      <c r="R85" t="n">
+        <v>0</v>
+      </c>
       <c r="S85" t="n">
         <v>0</v>
       </c>
@@ -43266,8 +43262,12 @@
       <c r="V85" t="n">
         <v>0</v>
       </c>
-      <c r="W85" t="inlineStr"/>
-      <c r="X85" t="inlineStr"/>
+      <c r="W85" t="n">
+        <v>0</v>
+      </c>
+      <c r="X85" t="n">
+        <v>0</v>
+      </c>
       <c r="Y85" t="inlineStr"/>
       <c r="Z85" t="inlineStr"/>
       <c r="AA85" t="inlineStr"/>
@@ -43275,12 +43275,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Lauberbach</t>
+          <t>Lisman</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -43336,7 +43336,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>De Martis</t>
+          <t>Lauberbach</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -43346,7 +43346,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -43394,8 +43394,69 @@
       <c r="Z87" t="inlineStr"/>
       <c r="AA87" t="inlineStr"/>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>De Martis</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Pc</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>Scommessa</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
+      <c r="P88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr"/>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="n">
+        <v>0</v>
+      </c>
+      <c r="T88" t="n">
+        <v>0</v>
+      </c>
+      <c r="U88" t="n">
+        <v>0</v>
+      </c>
+      <c r="V88" t="n">
+        <v>0</v>
+      </c>
+      <c r="W88" t="inlineStr"/>
+      <c r="X88" t="inlineStr"/>
+      <c r="Y88" t="inlineStr"/>
+      <c r="Z88" t="inlineStr"/>
+      <c r="AA88" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA87"/>
+  <autoFilter ref="A1:AA88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-08-27
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Portieri'!$A$1:$AA$63</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Difensori'!$A$1:$AA$185</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Centrocampisti'!$A$1:$AA$185</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Attaccanti'!$A$1:$AA$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Attaccanti'!$A$1:$AA$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33941,7 +33941,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -36118,7 +36118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA87"/>
+  <dimension ref="A1:AA88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -37735,27 +37735,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Simeone</t>
+          <t>Raspadori</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E19" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F19" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
@@ -37763,36 +37763,36 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>60.1</v>
+        <v>60.5</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Trappola</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="K19" t="n">
-        <v>6.08</v>
+        <v>6.12</v>
       </c>
       <c r="L19" t="n">
-        <v>7.09</v>
+        <v>6.88</v>
       </c>
       <c r="M19" t="n">
         <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>1.09</v>
+        <v>-0.05</v>
       </c>
       <c r="O19" t="n">
-        <v>0.596</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="P19" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
@@ -37801,16 +37801,16 @@
         <v>1</v>
       </c>
       <c r="T19" t="n">
-        <v>5.5</v>
+        <v>10</v>
       </c>
       <c r="U19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V19" t="n">
         <v>0</v>
       </c>
       <c r="W19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X19" t="n">
         <v>0</v>
@@ -37822,73 +37822,73 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Leao</t>
+          <t>Simeone</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E20" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F20" t="n">
-        <v>38</v>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>2a Fascia</t>
+        <v>40</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>1a Fascia</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>84.3</v>
+        <v>60.1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Trappola</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="K20" t="n">
-        <v>5.88</v>
+        <v>6.08</v>
       </c>
       <c r="L20" t="n">
-        <v>6.86</v>
+        <v>7.09</v>
       </c>
       <c r="M20" t="n">
         <v>3</v>
       </c>
       <c r="N20" t="n">
-        <v>-0.33</v>
+        <v>1.09</v>
       </c>
       <c r="O20" t="n">
-        <v>0.833</v>
+        <v>0.596</v>
       </c>
       <c r="P20" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -37897,7 +37897,7 @@
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="X20" t="n">
         <v>0</v>
@@ -37909,7 +37909,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Esposito Se.</t>
+          <t>Leao</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -37919,17 +37919,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E21" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="F21" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -37937,39 +37937,39 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>77.90000000000001</v>
+        <v>84.3</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Affare</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="K21" t="n">
-        <v>6.26</v>
+        <v>5.88</v>
       </c>
       <c r="L21" t="n">
-        <v>6.88</v>
+        <v>6.86</v>
       </c>
       <c r="M21" t="n">
         <v>3</v>
       </c>
       <c r="N21" t="n">
-        <v>2.64</v>
+        <v>-0.33</v>
       </c>
       <c r="O21" t="n">
-        <v>0.605</v>
+        <v>0.833</v>
       </c>
       <c r="P21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S21" t="n">
         <v>0</v>
@@ -37984,7 +37984,7 @@
         <v>0</v>
       </c>
       <c r="W21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X21" t="n">
         <v>0</v>
@@ -37996,7 +37996,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Soulè</t>
+          <t>Esposito Se.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -38006,17 +38006,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E22" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F22" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
@@ -38024,54 +38024,54 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>76.8</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Affare</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="K22" t="n">
-        <v>6.12</v>
+        <v>6.26</v>
       </c>
       <c r="L22" t="n">
-        <v>6.83</v>
+        <v>6.88</v>
       </c>
       <c r="M22" t="n">
         <v>3</v>
       </c>
       <c r="N22" t="n">
-        <v>-0.22</v>
+        <v>2.64</v>
       </c>
       <c r="O22" t="n">
-        <v>0.798</v>
+        <v>0.605</v>
       </c>
       <c r="P22" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>4</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="n">
         <v>6</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>5</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" t="n">
-        <v>1</v>
-      </c>
-      <c r="T22" t="n">
-        <v>6</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" t="n">
-        <v>0</v>
-      </c>
-      <c r="W22" t="n">
-        <v>1</v>
       </c>
       <c r="X22" t="n">
         <v>0</v>
@@ -38083,27 +38083,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pinamonti</t>
+          <t>Soulè</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E23" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F23" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -38111,7 +38111,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>74.59999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -38119,37 +38119,37 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="K23" t="n">
-        <v>5.88</v>
+        <v>6.12</v>
       </c>
       <c r="L23" t="n">
-        <v>6.62</v>
+        <v>6.83</v>
       </c>
       <c r="M23" t="n">
         <v>3</v>
       </c>
       <c r="N23" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.22</v>
       </c>
       <c r="O23" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.798</v>
       </c>
       <c r="P23" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Q23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -38158,10 +38158,10 @@
         <v>0</v>
       </c>
       <c r="W23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
@@ -38170,27 +38170,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Adams C.</t>
+          <t>Pinamonti</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E24" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="F24" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
@@ -38198,57 +38198,57 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>72.09999999999999</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Affare</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K24" t="n">
-        <v>5.98</v>
+        <v>5.88</v>
       </c>
       <c r="L24" t="n">
-        <v>6.64</v>
+        <v>6.62</v>
       </c>
       <c r="M24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N24" t="n">
-        <v>-0.12</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="O24" t="n">
-        <v>0.882</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="P24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="Q24" t="n">
         <v>3</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T24" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
@@ -38257,27 +38257,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dovbyk</t>
+          <t>Adams C.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="F25" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
@@ -38285,37 +38285,37 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>64</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Affare</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="K25" t="n">
-        <v>6</v>
+        <v>5.98</v>
       </c>
       <c r="L25" t="n">
-        <v>6.77</v>
+        <v>6.64</v>
       </c>
       <c r="M25" t="n">
         <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>-0.42</v>
+        <v>-0.12</v>
       </c>
       <c r="O25" t="n">
-        <v>0.592</v>
+        <v>0.882</v>
       </c>
       <c r="P25" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q25" t="n">
         <v>3</v>
       </c>
-      <c r="Q25" t="n">
-        <v>1</v>
-      </c>
       <c r="R25" t="n">
         <v>0</v>
       </c>
@@ -38323,10 +38323,10 @@
         <v>1</v>
       </c>
       <c r="T25" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V25" t="n">
         <v>0</v>
@@ -38344,7 +38344,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Castro S.</t>
+          <t>Dovbyk</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -38354,17 +38354,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E26" t="n">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="F26" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
@@ -38372,7 +38372,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>61.8</v>
+        <v>64</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -38380,26 +38380,26 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="K26" t="n">
-        <v>5.93</v>
+        <v>6</v>
       </c>
       <c r="L26" t="n">
-        <v>6.51</v>
+        <v>6.77</v>
       </c>
       <c r="M26" t="n">
+        <v>2</v>
+      </c>
+      <c r="N26" t="n">
+        <v>-0.42</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.592</v>
+      </c>
+      <c r="P26" t="n">
         <v>3</v>
       </c>
-      <c r="N26" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="P26" t="n">
-        <v>7</v>
-      </c>
       <c r="Q26" t="n">
         <v>1</v>
       </c>
@@ -38410,7 +38410,7 @@
         <v>1</v>
       </c>
       <c r="T26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -38419,7 +38419,7 @@
         <v>0</v>
       </c>
       <c r="W26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X26" t="n">
         <v>0</v>
@@ -38431,7 +38431,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pellegrino M.</t>
+          <t>Castro S.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -38441,17 +38441,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>14</v>
       </c>
       <c r="E27" t="n">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="F27" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
@@ -38459,7 +38459,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>60.6</v>
+        <v>61.8</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -38467,37 +38467,37 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K27" t="n">
-        <v>5.99</v>
+        <v>5.93</v>
       </c>
       <c r="L27" t="n">
-        <v>6.65</v>
+        <v>6.51</v>
       </c>
       <c r="M27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N27" t="n">
-        <v>-0.21</v>
+        <v>-0.15</v>
       </c>
       <c r="O27" t="n">
-        <v>0.632</v>
+        <v>0.64</v>
       </c>
       <c r="P27" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
         <v>1</v>
       </c>
       <c r="T27" t="n">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -38506,7 +38506,7 @@
         <v>0</v>
       </c>
       <c r="W27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="X27" t="n">
         <v>0</v>
@@ -38518,27 +38518,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Raspadori</t>
+          <t>Pellegrino M.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D28" t="n">
         <v>14</v>
       </c>
       <c r="E28" t="n">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="F28" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
@@ -38546,7 +38546,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>60.5</v>
+        <v>60.6</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -38554,46 +38554,46 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="K28" t="n">
-        <v>6.12</v>
+        <v>5.99</v>
       </c>
       <c r="L28" t="n">
-        <v>6.88</v>
+        <v>6.65</v>
       </c>
       <c r="M28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N28" t="n">
-        <v>-0.05</v>
+        <v>-0.21</v>
       </c>
       <c r="O28" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.632</v>
       </c>
       <c r="P28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="Q28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S28" t="n">
         <v>1</v>
       </c>
       <c r="T28" t="n">
-        <v>10</v>
+        <v>4.5</v>
       </c>
       <c r="U28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V28" t="n">
         <v>0</v>
       </c>
       <c r="W28" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X28" t="n">
         <v>0</v>
@@ -41605,71 +41605,51 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Frigan</t>
+          <t>Geubbels</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E65" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F65" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
           <t>3a Fascia</t>
         </is>
       </c>
-      <c r="H65" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J65" t="n">
-        <v>0</v>
-      </c>
-      <c r="K65" t="n">
-        <v>0</v>
-      </c>
-      <c r="L65" t="n">
-        <v>0</v>
-      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
       <c r="M65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N65" t="inlineStr"/>
-      <c r="O65" t="n">
-        <v>0</v>
-      </c>
-      <c r="P65" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R65" t="n">
-        <v>0</v>
-      </c>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
       <c r="S65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T65" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
@@ -41677,12 +41657,8 @@
       <c r="V65" t="n">
         <v>0</v>
       </c>
-      <c r="W65" t="n">
-        <v>0</v>
-      </c>
-      <c r="X65" t="n">
-        <v>0</v>
-      </c>
+      <c r="W65" t="inlineStr"/>
+      <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr"/>
       <c r="Z65" t="inlineStr"/>
       <c r="AA65" t="inlineStr"/>
@@ -41690,7 +41666,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Geubbels</t>
+          <t>Rrahmani Al.</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -41700,17 +41676,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D66" t="n">
+        <v>8</v>
+      </c>
+      <c r="E66" t="n">
+        <v>18</v>
+      </c>
+      <c r="F66" t="n">
         <v>9</v>
-      </c>
-      <c r="E66" t="n">
-        <v>23</v>
-      </c>
-      <c r="F66" t="n">
-        <v>12</v>
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
@@ -41731,10 +41707,10 @@
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="U66" t="n">
         <v>0</v>
@@ -41751,7 +41727,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Rrahmani Al.</t>
+          <t>Adorante</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -41765,13 +41741,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E67" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F67" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
@@ -41812,27 +41788,27 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Adorante</t>
+          <t>Fatah</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E68" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F68" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
@@ -42816,60 +42792,84 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Varela G.</t>
+          <t>Frigan</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>5</v>
       </c>
       <c r="E80" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
           <t>Low Cost</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
+      <c r="H80" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
       <c r="M80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
-      <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
+      <c r="O80" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0</v>
+      </c>
       <c r="S80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="U80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V80" t="n">
         <v>0</v>
       </c>
-      <c r="W80" t="inlineStr"/>
-      <c r="X80" t="inlineStr"/>
+      <c r="W80" t="n">
+        <v>0</v>
+      </c>
+      <c r="X80" t="n">
+        <v>0</v>
+      </c>
       <c r="Y80" t="inlineStr"/>
       <c r="Z80" t="inlineStr"/>
       <c r="AA80" t="inlineStr"/>
@@ -42877,7 +42877,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Havel</t>
+          <t>Varela G.</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -42887,14 +42887,14 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E81" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F81" t="n">
         <v>4</v>
@@ -42918,13 +42918,13 @@
       <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T81" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V81" t="n">
         <v>0</v>
@@ -42938,27 +42938,27 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Robinson J.</t>
+          <t>Havel</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>4</v>
       </c>
       <c r="E82" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
@@ -42999,7 +42999,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Lontani</t>
+          <t>Robinson J.</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -43009,11 +43009,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E83" t="n">
         <v>10</v>
@@ -43040,10 +43040,10 @@
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr"/>
       <c r="S83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T83" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="U83" t="n">
         <v>0</v>
@@ -43060,73 +43060,51 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Azon</t>
+          <t>Lontani</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F84" t="n">
-        <v>1</v>
-      </c>
-      <c r="G84" s="7" t="inlineStr">
-        <is>
-          <t>Scommessa</t>
-        </is>
-      </c>
-      <c r="H84" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J84" t="n">
-        <v>0</v>
-      </c>
-      <c r="K84" t="n">
-        <v>0</v>
-      </c>
-      <c r="L84" t="n">
-        <v>0</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>Low Cost</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
       <c r="M84" t="n">
-        <v>2</v>
-      </c>
-      <c r="N84" t="n">
-        <v>0</v>
-      </c>
-      <c r="O84" t="n">
-        <v>0</v>
-      </c>
-      <c r="P84" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q84" t="n">
-        <v>0</v>
-      </c>
-      <c r="R84" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T84" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="U84" t="n">
         <v>0</v>
@@ -43134,12 +43112,8 @@
       <c r="V84" t="n">
         <v>0</v>
       </c>
-      <c r="W84" t="n">
-        <v>0</v>
-      </c>
-      <c r="X84" t="n">
-        <v>0</v>
-      </c>
+      <c r="W84" t="inlineStr"/>
+      <c r="X84" t="inlineStr"/>
       <c r="Y84" t="inlineStr"/>
       <c r="Z84" t="inlineStr"/>
       <c r="AA84" t="inlineStr"/>
@@ -43147,17 +43121,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Lisman</t>
+          <t>Azon</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>W;A</t>
+          <t>Pc</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -43174,19 +43148,41 @@
           <t>Scommessa</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
+      <c r="H85" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
       <c r="M85" t="n">
-        <v>0</v>
-      </c>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
-      <c r="P85" t="inlineStr"/>
-      <c r="Q85" t="inlineStr"/>
-      <c r="R85" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>0</v>
+      </c>
+      <c r="R85" t="n">
+        <v>0</v>
+      </c>
       <c r="S85" t="n">
         <v>0</v>
       </c>
@@ -43199,8 +43195,12 @@
       <c r="V85" t="n">
         <v>0</v>
       </c>
-      <c r="W85" t="inlineStr"/>
-      <c r="X85" t="inlineStr"/>
+      <c r="W85" t="n">
+        <v>0</v>
+      </c>
+      <c r="X85" t="n">
+        <v>0</v>
+      </c>
       <c r="Y85" t="inlineStr"/>
       <c r="Z85" t="inlineStr"/>
       <c r="AA85" t="inlineStr"/>
@@ -43208,12 +43208,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Lauberbach</t>
+          <t>Lisman</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Pc</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -43269,7 +43269,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>De Martis</t>
+          <t>Lauberbach</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -43279,7 +43279,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -43327,8 +43327,69 @@
       <c r="Z87" t="inlineStr"/>
       <c r="AA87" t="inlineStr"/>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>De Martis</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Pc</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="7" t="inlineStr">
+        <is>
+          <t>Scommessa</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
+      <c r="P88" t="inlineStr"/>
+      <c r="Q88" t="inlineStr"/>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="n">
+        <v>0</v>
+      </c>
+      <c r="T88" t="n">
+        <v>0</v>
+      </c>
+      <c r="U88" t="n">
+        <v>0</v>
+      </c>
+      <c r="V88" t="n">
+        <v>0</v>
+      </c>
+      <c r="W88" t="inlineStr"/>
+      <c r="X88" t="inlineStr"/>
+      <c r="Y88" t="inlineStr"/>
+      <c r="Z88" t="inlineStr"/>
+      <c r="AA88" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA87"/>
+  <autoFilter ref="A1:AA88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-09-06
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -704,10 +704,10 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T2" t="n">
-        <v>6.75</v>
+        <v>6.17</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -878,10 +878,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T4" t="n">
-        <v>6.25</v>
+        <v>5.83</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -965,10 +965,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T5" t="n">
-        <v>5.5</v>
+        <v>5.17</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -1200,10 +1200,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T8" t="n">
-        <v>1.75</v>
+        <v>2.5</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1287,10 +1287,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" t="n">
-        <v>5</v>
+        <v>4.67</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1872,10 +1872,10 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T16" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -5959,16 +5959,16 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T2" t="n">
-        <v>6.25</v>
+        <v>6.67</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W2" t="n">
         <v>3</v>
@@ -6046,10 +6046,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T3" t="n">
-        <v>7</v>
+        <v>6.33</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -6218,10 +6218,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T5" t="n">
-        <v>7.25</v>
+        <v>7.17</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -6392,10 +6392,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T7" t="n">
-        <v>6.75</v>
+        <v>6.33</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -6457,7 +6457,7 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T8" t="n">
         <v>6</v>
@@ -6540,10 +6540,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" t="n">
-        <v>5.75</v>
+        <v>5.67</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -6627,13 +6627,13 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" t="n">
-        <v>6.25</v>
+        <v>7.5</v>
       </c>
       <c r="U10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V10" t="n">
         <v>0</v>
@@ -6714,10 +6714,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T11" t="n">
-        <v>8.25</v>
+        <v>7.67</v>
       </c>
       <c r="U11" t="n">
         <v>1</v>
@@ -6801,16 +6801,16 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T12" t="n">
-        <v>5.75</v>
+        <v>6.17</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W12" t="n">
         <v>1</v>
@@ -6975,10 +6975,10 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" t="n">
-        <v>6</v>
+        <v>6.17</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -7149,10 +7149,10 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T16" t="n">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -7234,16 +7234,16 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T17" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W17" t="n">
         <v>4</v>
@@ -7408,10 +7408,10 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T19" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -8803,10 +8803,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T36" t="n">
-        <v>6</v>
+        <v>5.83</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -9151,16 +9151,16 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T40" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="U40" t="n">
         <v>0</v>
       </c>
       <c r="V40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W40" t="n">
         <v>6</v>
@@ -9236,16 +9236,16 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T41" t="n">
-        <v>3.75</v>
+        <v>4.67</v>
       </c>
       <c r="U41" t="n">
         <v>0</v>
       </c>
       <c r="V41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W41" t="n">
         <v>1</v>
@@ -9839,16 +9839,16 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T48" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="U48" t="n">
         <v>0</v>
       </c>
       <c r="V48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W48" t="n">
         <v>6</v>
@@ -10274,10 +10274,10 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T53" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U53" t="n">
         <v>0</v>
@@ -10446,10 +10446,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T55" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U55" t="n">
         <v>0</v>
@@ -10968,7 +10968,7 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T61" t="n">
         <v>6</v>
@@ -11142,10 +11142,10 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T63" t="n">
-        <v>7.75</v>
+        <v>7.17</v>
       </c>
       <c r="U63" t="n">
         <v>1</v>
@@ -12370,10 +12370,10 @@
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T79" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U79" t="n">
         <v>0</v>
@@ -12736,7 +12736,7 @@
       <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T85" t="n">
         <v>5</v>
@@ -13920,10 +13920,10 @@
         <v>0</v>
       </c>
       <c r="S99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T99" t="n">
-        <v>5</v>
+        <v>5.25</v>
       </c>
       <c r="U99" t="n">
         <v>0</v>
@@ -14268,10 +14268,10 @@
         <v>0</v>
       </c>
       <c r="S103" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T103" t="n">
-        <v>5.75</v>
+        <v>5.67</v>
       </c>
       <c r="U103" t="n">
         <v>0</v>
@@ -14355,10 +14355,10 @@
         <v>0</v>
       </c>
       <c r="S104" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T104" t="n">
-        <v>6</v>
+        <v>6.17</v>
       </c>
       <c r="U104" t="n">
         <v>0</v>
@@ -14873,10 +14873,10 @@
         <v>0</v>
       </c>
       <c r="S110" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T110" t="n">
-        <v>6</v>
+        <v>6.17</v>
       </c>
       <c r="U110" t="n">
         <v>0</v>
@@ -15733,10 +15733,10 @@
         <v>0</v>
       </c>
       <c r="S120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T120" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="U120" t="n">
         <v>0</v>
@@ -16658,7 +16658,7 @@
       <c r="Q131" t="inlineStr"/>
       <c r="R131" t="inlineStr"/>
       <c r="S131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T131" t="n">
         <v>5.5</v>
@@ -16780,10 +16780,10 @@
       <c r="Q133" t="inlineStr"/>
       <c r="R133" t="inlineStr"/>
       <c r="S133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T133" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="U133" t="n">
         <v>0</v>
@@ -16963,10 +16963,10 @@
       <c r="Q136" t="inlineStr"/>
       <c r="R136" t="inlineStr"/>
       <c r="S136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T136" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U136" t="n">
         <v>0</v>
@@ -17085,16 +17085,16 @@
       <c r="Q138" t="inlineStr"/>
       <c r="R138" t="inlineStr"/>
       <c r="S138" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T138" t="n">
-        <v>6</v>
+        <v>6.75</v>
       </c>
       <c r="U138" t="n">
         <v>0</v>
       </c>
       <c r="V138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr"/>
@@ -17329,10 +17329,10 @@
       <c r="Q142" t="inlineStr"/>
       <c r="R142" t="inlineStr"/>
       <c r="S142" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T142" t="n">
-        <v>6.5</v>
+        <v>6.33</v>
       </c>
       <c r="U142" t="n">
         <v>0</v>
@@ -18620,10 +18620,10 @@
         <v>0</v>
       </c>
       <c r="S157" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T157" t="n">
-        <v>5.25</v>
+        <v>5.17</v>
       </c>
       <c r="U157" t="n">
         <v>0</v>
@@ -21612,10 +21612,10 @@
         <v>5</v>
       </c>
       <c r="S5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T5" t="n">
-        <v>9.75</v>
+        <v>8.5</v>
       </c>
       <c r="U5" t="n">
         <v>2</v>
@@ -21956,10 +21956,10 @@
         <v>3</v>
       </c>
       <c r="S9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U9" t="n">
         <v>1</v>
@@ -22021,10 +22021,10 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" t="n">
-        <v>8.25</v>
+        <v>7.5</v>
       </c>
       <c r="U10" t="n">
         <v>1</v>
@@ -22191,10 +22191,10 @@
         <v>5</v>
       </c>
       <c r="S12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T12" t="n">
-        <v>5.25</v>
+        <v>5.33</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -22365,10 +22365,10 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -22887,10 +22887,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T20" t="n">
-        <v>5.25</v>
+        <v>5.33</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -22974,13 +22974,13 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T21" t="n">
-        <v>5.25</v>
+        <v>6.67</v>
       </c>
       <c r="U21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V21" t="n">
         <v>0</v>
@@ -23146,10 +23146,10 @@
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T23" t="n">
-        <v>8.25</v>
+        <v>7.67</v>
       </c>
       <c r="U23" t="n">
         <v>1</v>
@@ -23318,10 +23318,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T25" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -23492,13 +23492,13 @@
         <v>1</v>
       </c>
       <c r="S27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T27" t="n">
-        <v>5.75</v>
+        <v>7.17</v>
       </c>
       <c r="U27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V27" t="n">
         <v>0</v>
@@ -23664,10 +23664,10 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T29" t="n">
-        <v>6.25</v>
+        <v>6.17</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -23838,10 +23838,10 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T31" t="n">
-        <v>8</v>
+        <v>7.33</v>
       </c>
       <c r="U31" t="n">
         <v>1</v>
@@ -24010,10 +24010,10 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T33" t="n">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
@@ -24075,7 +24075,7 @@
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T34" t="n">
         <v>6</v>
@@ -24319,10 +24319,10 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T38" t="n">
-        <v>5.25</v>
+        <v>5.33</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -24550,13 +24550,13 @@
         <v>1</v>
       </c>
       <c r="S41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T41" t="n">
-        <v>5.25</v>
+        <v>7</v>
       </c>
       <c r="U41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V41" t="n">
         <v>0</v>
@@ -25151,7 +25151,7 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T48" t="n">
         <v>5.5</v>
@@ -25238,10 +25238,10 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T49" t="n">
-        <v>6.25</v>
+        <v>5.67</v>
       </c>
       <c r="U49" t="n">
         <v>0</v>
@@ -25673,10 +25673,10 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T54" t="n">
-        <v>6.5</v>
+        <v>6.33</v>
       </c>
       <c r="U54" t="n">
         <v>0</v>
@@ -26280,10 +26280,10 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T61" t="n">
-        <v>6.5</v>
+        <v>6.17</v>
       </c>
       <c r="U61" t="n">
         <v>0</v>
@@ -26367,10 +26367,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T62" t="n">
-        <v>6.75</v>
+        <v>6.33</v>
       </c>
       <c r="U62" t="n">
         <v>0</v>
@@ -26454,7 +26454,7 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T63" t="n">
         <v>5.5</v>
@@ -26541,10 +26541,10 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T64" t="n">
-        <v>5.25</v>
+        <v>5.33</v>
       </c>
       <c r="U64" t="n">
         <v>0</v>
@@ -26887,10 +26887,10 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T68" t="n">
-        <v>11.5</v>
+        <v>8.25</v>
       </c>
       <c r="U68" t="n">
         <v>1</v>
@@ -27235,10 +27235,10 @@
         <v>0</v>
       </c>
       <c r="S72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T72" t="n">
-        <v>6.25</v>
+        <v>6.33</v>
       </c>
       <c r="U72" t="n">
         <v>0</v>
@@ -27409,10 +27409,10 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T74" t="n">
-        <v>5</v>
+        <v>5.17</v>
       </c>
       <c r="U74" t="n">
         <v>0</v>
@@ -27583,10 +27583,10 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T76" t="n">
-        <v>6.5</v>
+        <v>6.25</v>
       </c>
       <c r="U76" t="n">
         <v>0</v>
@@ -27668,7 +27668,7 @@
         <v>0</v>
       </c>
       <c r="S77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T77" t="n">
         <v>6.5</v>
@@ -28334,10 +28334,10 @@
       <c r="Q87" t="inlineStr"/>
       <c r="R87" t="inlineStr"/>
       <c r="S87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T87" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U87" t="n">
         <v>0</v>
@@ -28765,10 +28765,10 @@
         <v>0</v>
       </c>
       <c r="S92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T92" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U92" t="n">
         <v>0</v>
@@ -31106,10 +31106,10 @@
         <v>0</v>
       </c>
       <c r="S119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T119" t="n">
-        <v>5.75</v>
+        <v>5.67</v>
       </c>
       <c r="U119" t="n">
         <v>0</v>
@@ -32637,10 +32637,10 @@
       <c r="Q138" t="inlineStr"/>
       <c r="R138" t="inlineStr"/>
       <c r="S138" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T138" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U138" t="n">
         <v>0</v>
@@ -32820,10 +32820,10 @@
       <c r="Q141" t="inlineStr"/>
       <c r="R141" t="inlineStr"/>
       <c r="S141" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T141" t="n">
-        <v>6</v>
+        <v>6.17</v>
       </c>
       <c r="U141" t="n">
         <v>0</v>
@@ -37140,13 +37140,13 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T2" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V2" t="n">
         <v>0</v>
@@ -37227,13 +37227,13 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T3" t="n">
-        <v>5.5</v>
+        <v>7.75</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
@@ -37312,13 +37312,13 @@
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T4" t="n">
-        <v>7.75</v>
+        <v>8.5</v>
       </c>
       <c r="U4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V4" t="n">
         <v>0</v>
@@ -37397,10 +37397,10 @@
         <v>4</v>
       </c>
       <c r="S5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T5" t="n">
-        <v>15.5</v>
+        <v>12.33</v>
       </c>
       <c r="U5" t="n">
         <v>5</v>
@@ -37545,10 +37545,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T7" t="n">
-        <v>7.5</v>
+        <v>6.67</v>
       </c>
       <c r="U7" t="n">
         <v>1</v>
@@ -37719,10 +37719,10 @@
         <v>2</v>
       </c>
       <c r="S9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -37978,10 +37978,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U12" t="n">
         <v>1</v>
@@ -38324,16 +38324,16 @@
         <v>1</v>
       </c>
       <c r="S16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T16" t="n">
-        <v>9</v>
+        <v>8.67</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W16" t="n">
         <v>0</v>
@@ -38498,10 +38498,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T18" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -38733,16 +38733,16 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T21" t="n">
-        <v>8</v>
+        <v>9.17</v>
       </c>
       <c r="U21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W21" t="n">
         <v>1</v>
@@ -38907,13 +38907,13 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T23" t="n">
-        <v>8</v>
+        <v>8.67</v>
       </c>
       <c r="U23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
@@ -39081,10 +39081,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T25" t="n">
-        <v>6</v>
+        <v>6.17</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -39255,13 +39255,13 @@
         <v>1</v>
       </c>
       <c r="S27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T27" t="n">
-        <v>4.5</v>
+        <v>6.17</v>
       </c>
       <c r="U27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V27" t="n">
         <v>0</v>
@@ -39342,10 +39342,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T28" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U28" t="n">
         <v>0</v>
@@ -39514,7 +39514,7 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T30" t="n">
         <v>6</v>
@@ -39945,10 +39945,10 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T35" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
@@ -40744,10 +40744,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T46" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -41090,10 +41090,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T50" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -42222,10 +42222,10 @@
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr"/>
       <c r="S64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T64" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U64" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-09-07
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -2275,10 +2275,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T21" t="n">
-        <v>4</v>
+        <v>3.67</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -2447,10 +2447,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T23" t="n">
-        <v>4.25</v>
+        <v>4.83</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2706,10 +2706,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T26" t="n">
-        <v>5.75</v>
+        <v>5.17</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -3004,10 +3004,10 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T30" t="n">
-        <v>1.5</v>
+        <v>3.25</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -7669,10 +7669,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T22" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -7841,10 +7841,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T24" t="n">
-        <v>6</v>
+        <v>6.17</v>
       </c>
       <c r="U24" t="n">
         <v>0</v>
@@ -8274,10 +8274,10 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T29" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -11401,10 +11401,10 @@
         <v>0</v>
       </c>
       <c r="S66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T66" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U66" t="n">
         <v>0</v>
@@ -11830,10 +11830,10 @@
         <v>0</v>
       </c>
       <c r="S71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T71" t="n">
-        <v>5.25</v>
+        <v>5.5</v>
       </c>
       <c r="U71" t="n">
         <v>0</v>
@@ -12248,10 +12248,10 @@
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T77" t="n">
-        <v>8.5</v>
+        <v>7.67</v>
       </c>
       <c r="U77" t="n">
         <v>1</v>
@@ -12309,16 +12309,16 @@
       <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T78" t="n">
-        <v>6.5</v>
+        <v>6.67</v>
       </c>
       <c r="U78" t="n">
         <v>0</v>
       </c>
       <c r="V78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -12797,10 +12797,10 @@
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T86" t="n">
-        <v>6</v>
+        <v>6.17</v>
       </c>
       <c r="U86" t="n">
         <v>0</v>
@@ -12965,10 +12965,10 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T88" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U88" t="n">
         <v>0</v>
@@ -13400,16 +13400,16 @@
         <v>0</v>
       </c>
       <c r="S93" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T93" t="n">
-        <v>5.75</v>
+        <v>6.33</v>
       </c>
       <c r="U93" t="n">
         <v>0</v>
       </c>
       <c r="V93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W93" t="n">
         <v>0</v>
@@ -14181,10 +14181,10 @@
         <v>0</v>
       </c>
       <c r="S102" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T102" t="n">
-        <v>5.75</v>
+        <v>5.67</v>
       </c>
       <c r="U102" t="n">
         <v>0</v>
@@ -14614,10 +14614,10 @@
         <v>0</v>
       </c>
       <c r="S107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T107" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U107" t="n">
         <v>0</v>
@@ -14788,10 +14788,10 @@
         <v>0</v>
       </c>
       <c r="S109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T109" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U109" t="n">
         <v>0</v>
@@ -15130,7 +15130,7 @@
         <v>0</v>
       </c>
       <c r="S113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T113" t="n">
         <v>6</v>
@@ -16079,16 +16079,16 @@
         <v>0</v>
       </c>
       <c r="S124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T124" t="n">
-        <v>6.25</v>
+        <v>6.67</v>
       </c>
       <c r="U124" t="n">
         <v>0</v>
       </c>
       <c r="V124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W124" t="n">
         <v>4</v>
@@ -16251,10 +16251,10 @@
         <v>0</v>
       </c>
       <c r="S126" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T126" t="n">
-        <v>5.25</v>
+        <v>5</v>
       </c>
       <c r="U126" t="n">
         <v>0</v>
@@ -16421,10 +16421,10 @@
         <v>0</v>
       </c>
       <c r="S128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T128" t="n">
-        <v>4.75</v>
+        <v>5.33</v>
       </c>
       <c r="U128" t="n">
         <v>0</v>
@@ -17207,10 +17207,10 @@
       <c r="Q140" t="inlineStr"/>
       <c r="R140" t="inlineStr"/>
       <c r="S140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T140" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="U140" t="n">
         <v>0</v>
@@ -18535,10 +18535,10 @@
         <v>0</v>
       </c>
       <c r="S156" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T156" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U156" t="n">
         <v>0</v>
@@ -19138,10 +19138,10 @@
         <v>0</v>
       </c>
       <c r="S163" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T163" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U163" t="n">
         <v>0</v>
@@ -19652,13 +19652,13 @@
         <v>0</v>
       </c>
       <c r="S169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T169" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V169" t="n">
         <v>0</v>
@@ -27907,10 +27907,10 @@
       <c r="Q80" t="inlineStr"/>
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T80" t="n">
-        <v>6.75</v>
+        <v>6.67</v>
       </c>
       <c r="U80" t="n">
         <v>0</v>
@@ -27968,7 +27968,7 @@
       <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T81" t="n">
         <v>5.5</v>
@@ -28591,10 +28591,10 @@
         <v>0</v>
       </c>
       <c r="S90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T90" t="n">
-        <v>7.25</v>
+        <v>6.83</v>
       </c>
       <c r="U90" t="n">
         <v>1</v>
@@ -30155,10 +30155,10 @@
         <v>0</v>
       </c>
       <c r="S108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T108" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="U108" t="n">
         <v>0</v>
@@ -30240,16 +30240,16 @@
         <v>0</v>
       </c>
       <c r="S109" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T109" t="n">
-        <v>5.75</v>
+        <v>6.17</v>
       </c>
       <c r="U109" t="n">
         <v>0</v>
       </c>
       <c r="V109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W109" t="n">
         <v>4</v>
@@ -30412,10 +30412,10 @@
         <v>0</v>
       </c>
       <c r="S111" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T111" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U111" t="n">
         <v>0</v>
@@ -30760,7 +30760,7 @@
         <v>0</v>
       </c>
       <c r="S115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T115" t="n">
         <v>5.5</v>
@@ -30932,10 +30932,10 @@
         <v>0</v>
       </c>
       <c r="S117" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T117" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="U117" t="n">
         <v>0</v>
@@ -31019,10 +31019,10 @@
         <v>0</v>
       </c>
       <c r="S118" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T118" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="U118" t="n">
         <v>0</v>
@@ -31620,10 +31620,10 @@
         <v>0</v>
       </c>
       <c r="S125" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T125" t="n">
-        <v>7.5</v>
+        <v>6.75</v>
       </c>
       <c r="U125" t="n">
         <v>0</v>
@@ -32304,7 +32304,7 @@
         <v>0</v>
       </c>
       <c r="S133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T133" t="n">
         <v>6</v>
@@ -32881,10 +32881,10 @@
       <c r="Q142" t="inlineStr"/>
       <c r="R142" t="inlineStr"/>
       <c r="S142" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T142" t="n">
-        <v>5.5</v>
+        <v>5.75</v>
       </c>
       <c r="U142" t="n">
         <v>0</v>
@@ -33578,10 +33578,10 @@
         <v>0</v>
       </c>
       <c r="S151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T151" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U151" t="n">
         <v>0</v>
@@ -34361,16 +34361,16 @@
         <v>0</v>
       </c>
       <c r="S160" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T160" t="n">
-        <v>6.25</v>
+        <v>6.67</v>
       </c>
       <c r="U160" t="n">
         <v>0</v>
       </c>
       <c r="V160" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W160" t="n">
         <v>5</v>
@@ -34620,10 +34620,10 @@
         <v>0</v>
       </c>
       <c r="S163" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T163" t="n">
-        <v>6</v>
+        <v>5.83</v>
       </c>
       <c r="U163" t="n">
         <v>0</v>
@@ -35926,10 +35926,10 @@
       <c r="Q179" t="inlineStr"/>
       <c r="R179" t="inlineStr"/>
       <c r="S179" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T179" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U179" t="n">
         <v>0</v>
@@ -35987,10 +35987,10 @@
       <c r="Q180" t="inlineStr"/>
       <c r="R180" t="inlineStr"/>
       <c r="S180" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T180" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U180" t="n">
         <v>0</v>
@@ -36336,10 +36336,10 @@
         <v>0</v>
       </c>
       <c r="S185" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T185" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="U185" t="n">
         <v>0</v>
@@ -39860,10 +39860,10 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T34" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U34" t="n">
         <v>0</v>
@@ -40032,13 +40032,13 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T36" t="n">
-        <v>9.5</v>
+        <v>10.83</v>
       </c>
       <c r="U36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V36" t="n">
         <v>0</v>
@@ -40158,7 +40158,7 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T38" t="n">
         <v>5.5</v>
@@ -40219,10 +40219,10 @@
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T39" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="U39" t="n">
         <v>0</v>
@@ -41519,13 +41519,13 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T55" t="n">
-        <v>6.25</v>
+        <v>7.5</v>
       </c>
       <c r="U55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V55" t="n">
         <v>0</v>
@@ -41950,10 +41950,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T60" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U60" t="n">
         <v>0</v>
@@ -42035,13 +42035,13 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T61" t="n">
-        <v>7.25</v>
+        <v>8.17</v>
       </c>
       <c r="U61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V61" t="n">
         <v>1</v>
@@ -42161,10 +42161,10 @@
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr"/>
       <c r="S63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T63" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U63" t="n">
         <v>0</v>
@@ -42466,13 +42466,13 @@
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T68" t="n">
-        <v>6.25</v>
+        <v>7.5</v>
       </c>
       <c r="U68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V68" t="n">
         <v>0</v>
@@ -42634,10 +42634,10 @@
         <v>0</v>
       </c>
       <c r="S70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T70" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U70" t="n">
         <v>0</v>
@@ -43320,10 +43320,10 @@
         <v>0</v>
       </c>
       <c r="S78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T78" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U78" t="n">
         <v>0</v>
@@ -43507,13 +43507,13 @@
       <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T81" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V81" t="n">
         <v>0</v>
@@ -43836,10 +43836,10 @@
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T86" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U86" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-09-10
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Attaccanti" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Portieri'!$A$1:$AA$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Portieri'!$A$1:$AA$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Difensori'!$A$1:$AA$191</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Centrocampisti'!$A$1:$AA$193</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Attaccanti'!$A$1:$AA$87</definedName>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA65"/>
+  <dimension ref="A1:AA64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>70.3</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>71.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>71.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>69.3</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>68.40000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>68.2</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1600,7 +1600,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>59.2</v>
+        <v>58.8</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>59.2</v>
+        <v>58.7</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Muric</t>
+          <t>Perri</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1756,61 +1756,41 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
           <t>1a Fascia</t>
         </is>
       </c>
-      <c r="H15" t="n">
-        <v>57.6</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Trappola</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>32</v>
-      </c>
-      <c r="K15" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="L15" t="n">
-        <v>4.77</v>
-      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15" t="inlineStr"/>
-      <c r="O15" t="n">
-        <v>0.842</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
-      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T15" t="n">
-        <v>4.33</v>
+        <v>4.5</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -1818,12 +1798,8 @@
       <c r="V15" t="n">
         <v>0</v>
       </c>
-      <c r="W15" t="n">
-        <v>43</v>
-      </c>
-      <c r="X15" t="n">
-        <v>1</v>
-      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
@@ -1831,7 +1807,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Perri</t>
+          <t>Sanchez Ro.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1841,17 +1817,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F16" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
@@ -1872,10 +1848,10 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -1892,7 +1868,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sanchez Ro.</t>
+          <t>Milinkovic-Savic V.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1902,36 +1878,58 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
-        <v>8</v>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>1a Fascia</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>2a Fascia</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Affare</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>27</v>
+      </c>
+      <c r="K17" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="L17" t="n">
+        <v>5.65</v>
+      </c>
       <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
       <c r="S17" t="n">
         <v>0</v>
       </c>
@@ -1944,8 +1942,12 @@
       <c r="V17" t="n">
         <v>0</v>
       </c>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
+      <c r="W17" t="n">
+        <v>24</v>
+      </c>
+      <c r="X17" t="n">
+        <v>3</v>
+      </c>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr"/>
@@ -1953,7 +1955,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Milinkovic-Savic V.</t>
+          <t>Pessina Mas.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1963,48 +1965,46 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>2a Fascia</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Affare</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
         <v>4</v>
       </c>
-      <c r="E18" t="n">
-        <v>5</v>
-      </c>
-      <c r="F18" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>2a Fascia</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>83.3</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Affare</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>27</v>
-      </c>
       <c r="K18" t="n">
-        <v>6.2</v>
+        <v>6.12</v>
       </c>
       <c r="L18" t="n">
-        <v>5.65</v>
+        <v>5.62</v>
       </c>
       <c r="M18" t="n">
-        <v>3</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0.28</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
-        <v>0.877</v>
+        <v>0.105</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -2028,10 +2028,10 @@
         <v>0</v>
       </c>
       <c r="W18" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr"/>
@@ -2040,7 +2040,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pessina Mas.</t>
+          <t>Provedel</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2050,17 +2050,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
@@ -2068,28 +2068,30 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>68.8</v>
+        <v>63.3</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Affare</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="K19" t="n">
-        <v>6.12</v>
+        <v>6.26</v>
       </c>
       <c r="L19" t="n">
-        <v>5.62</v>
+        <v>5.35</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N19" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.59</v>
+      </c>
       <c r="O19" t="n">
-        <v>0.105</v>
+        <v>0.754</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -2113,10 +2115,10 @@
         <v>0</v>
       </c>
       <c r="W19" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
@@ -2125,7 +2127,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Provedel</t>
+          <t>Stankovic F.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2135,17 +2137,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
@@ -2153,7 +2155,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>63.6</v>
+        <v>61.3</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2161,22 +2163,22 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="K20" t="n">
-        <v>6.26</v>
+        <v>6.6</v>
       </c>
       <c r="L20" t="n">
-        <v>5.35</v>
+        <v>5.23</v>
       </c>
       <c r="M20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N20" t="n">
-        <v>0.59</v>
+        <v>5.23</v>
       </c>
       <c r="O20" t="n">
-        <v>0.754</v>
+        <v>0.197</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -2188,10 +2190,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>3.67</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -2200,7 +2202,7 @@
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="X20" t="n">
         <v>1</v>
@@ -2212,7 +2214,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Stankovic F.</t>
+          <t>Muric</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2222,17 +2224,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
@@ -2240,30 +2242,28 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>61.7</v>
+        <v>57.1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Trappola</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="K21" t="n">
-        <v>6.6</v>
+        <v>6.08</v>
       </c>
       <c r="L21" t="n">
-        <v>5.23</v>
+        <v>4.77</v>
       </c>
       <c r="M21" t="n">
-        <v>2</v>
-      </c>
-      <c r="N21" t="n">
-        <v>5.23</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="n">
-        <v>0.197</v>
+        <v>0.842</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
@@ -2278,7 +2278,7 @@
         <v>3</v>
       </c>
       <c r="T21" t="n">
-        <v>3.67</v>
+        <v>4.33</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -2287,7 +2287,7 @@
         <v>0</v>
       </c>
       <c r="W21" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="X21" t="n">
         <v>1</v>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>56</v>
+        <v>55.7</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -2414,7 +2414,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>48.1</v>
+        <v>47.6</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Christensen O.</t>
+          <t>Sportiello</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -2499,7 +2499,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>42.3</v>
+        <v>36.8</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2510,19 +2510,19 @@
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="L24" t="n">
-        <v>6.5</v>
+        <v>4.5</v>
       </c>
       <c r="M24" t="n">
         <v>3</v>
       </c>
       <c r="N24" t="n">
-        <v>5.28</v>
+        <v>-0.34</v>
       </c>
       <c r="O24" t="n">
-        <v>0.044</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
@@ -2558,7 +2558,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sportiello</t>
+          <t>Sherri</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>37.6</v>
+        <v>34.1</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2594,22 +2594,22 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>-0.34</v>
+        <v>-4.29</v>
       </c>
       <c r="O25" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.092</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -2633,7 +2633,7 @@
         <v>0</v>
       </c>
       <c r="W25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X25" t="n">
         <v>0</v>
@@ -2645,7 +2645,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sherri</t>
+          <t>Palmisani</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2655,17 +2655,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
@@ -2673,11 +2673,11 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>34.9</v>
+        <v>30.8</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Trappola</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -2690,13 +2690,11 @@
         <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>2</v>
-      </c>
-      <c r="N26" t="n">
-        <v>-4.29</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="n">
-        <v>0.092</v>
+        <v>0</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2708,10 +2706,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T26" t="n">
-        <v>0</v>
+        <v>5.17</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -2732,7 +2730,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Palmisani</t>
+          <t>Tornqvist</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2742,25 +2740,25 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" t="n">
         <v>5</v>
       </c>
-      <c r="E27" t="n">
-        <v>12</v>
-      </c>
-      <c r="F27" t="n">
-        <v>6</v>
-      </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
           <t>2a Fascia</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2793,10 +2791,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>5.17</v>
+        <v>0</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -2817,7 +2815,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tornqvist</t>
+          <t>Vigorito</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2827,17 +2825,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
@@ -2845,11 +2843,11 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Trappola</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -2862,9 +2860,11 @@
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
-      </c>
-      <c r="N28" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
@@ -2902,7 +2902,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Vigorito</t>
+          <t>Daffara</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2912,58 +2912,36 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
           <t>2a Fascia</t>
         </is>
       </c>
-      <c r="H29" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
-        <v>2</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
       <c r="S29" t="n">
         <v>0</v>
       </c>
@@ -2976,12 +2954,8 @@
       <c r="V29" t="n">
         <v>0</v>
       </c>
-      <c r="W29" t="n">
-        <v>0</v>
-      </c>
-      <c r="X29" t="n">
-        <v>0</v>
-      </c>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="inlineStr"/>
@@ -2989,7 +2963,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Daffara</t>
+          <t>Thiam</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2999,17 +2973,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
@@ -3030,10 +3004,10 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T30" t="n">
-        <v>0</v>
+        <v>3.25</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -3050,7 +3024,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Thiam</t>
+          <t>Happonen</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3060,17 +3034,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
@@ -3091,10 +3065,10 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T31" t="n">
-        <v>3.25</v>
+        <v>0</v>
       </c>
       <c r="U31" t="n">
         <v>0</v>
@@ -3111,7 +3085,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Happonen</t>
+          <t>Mascardi</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3121,17 +3095,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D32" t="n">
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
@@ -3152,10 +3126,10 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T32" t="n">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="U32" t="n">
         <v>0</v>
@@ -3172,7 +3146,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mascardi</t>
+          <t>Terracciano</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3182,41 +3156,63 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>2a Fascia</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>3a Fascia</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Affare</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" t="n">
+        <v>6</v>
+      </c>
+      <c r="L33" t="n">
+        <v>6</v>
+      </c>
       <c r="M33" t="n">
-        <v>0</v>
-      </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0</v>
+      </c>
       <c r="S33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T33" t="n">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
@@ -3224,8 +3220,12 @@
       <c r="V33" t="n">
         <v>0</v>
       </c>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
+      <c r="W33" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" t="n">
+        <v>0</v>
+      </c>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
       <c r="AA33" t="inlineStr"/>
@@ -3233,7 +3233,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Terracciano</t>
+          <t>Motta</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -3261,7 +3261,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>73.90000000000001</v>
+        <v>62.8</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -3269,22 +3269,20 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K34" t="n">
         <v>6</v>
       </c>
       <c r="L34" t="n">
-        <v>6</v>
+        <v>5.17</v>
       </c>
       <c r="M34" t="n">
-        <v>3</v>
-      </c>
-      <c r="N34" t="n">
-        <v>0.8</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N34" t="inlineStr"/>
       <c r="O34" t="n">
-        <v>0.333</v>
+        <v>0.237</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
@@ -3308,10 +3306,10 @@
         <v>0</v>
       </c>
       <c r="W34" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y34" t="inlineStr"/>
       <c r="Z34" t="inlineStr"/>
@@ -3320,7 +3318,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Motta</t>
+          <t>Turati</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3330,7 +3328,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -3348,7 +3346,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>63.2</v>
+        <v>53.2</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -3356,20 +3354,22 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K35" t="n">
-        <v>6</v>
+        <v>6.17</v>
       </c>
       <c r="L35" t="n">
-        <v>5.17</v>
+        <v>5</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
-      </c>
-      <c r="N35" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.37</v>
+      </c>
       <c r="O35" t="n">
-        <v>0.237</v>
+        <v>0.588</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
@@ -3393,10 +3393,10 @@
         <v>0</v>
       </c>
       <c r="W35" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="X35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
@@ -3405,7 +3405,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Turati</t>
+          <t>Christensen O.</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -3433,30 +3433,30 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>53.8</v>
+        <v>41.7</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Affare</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K36" t="n">
-        <v>6.17</v>
+        <v>7.5</v>
       </c>
       <c r="L36" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="M36" t="n">
         <v>3</v>
       </c>
       <c r="N36" t="n">
-        <v>0.37</v>
+        <v>5.28</v>
       </c>
       <c r="O36" t="n">
-        <v>0.588</v>
+        <v>0.044</v>
       </c>
       <c r="P36" t="n">
         <v>0</v>
@@ -3480,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="W36" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="X36" t="n">
         <v>0</v>
@@ -3492,7 +3492,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Padelli</t>
+          <t>Pinsoglio</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -3520,30 +3520,30 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>48.2</v>
+        <v>41.4</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Affare</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>5.25</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
         <v>3</v>
       </c>
       <c r="N37" t="n">
-        <v>1.19</v>
+        <v>-2.44</v>
       </c>
       <c r="O37" t="n">
-        <v>0.026</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="P37" t="n">
         <v>0</v>
@@ -3567,7 +3567,7 @@
         <v>0</v>
       </c>
       <c r="W37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X37" t="n">
         <v>0</v>
@@ -3579,7 +3579,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Pinsoglio</t>
+          <t>Contini</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>42.3</v>
+        <v>40.5</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -3627,7 +3627,7 @@
         <v>3</v>
       </c>
       <c r="N38" t="n">
-        <v>-2.44</v>
+        <v>-2.25</v>
       </c>
       <c r="O38" t="n">
         <v>0.008999999999999999</v>
@@ -3666,7 +3666,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Contini</t>
+          <t>Di Gennaro</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -3694,7 +3694,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>41.4</v>
+        <v>40</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -3702,22 +3702,22 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L39" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M39" t="n">
         <v>3</v>
       </c>
       <c r="N39" t="n">
-        <v>-2.25</v>
+        <v>2.56</v>
       </c>
       <c r="O39" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.018</v>
       </c>
       <c r="P39" t="n">
         <v>0</v>
@@ -3741,7 +3741,7 @@
         <v>0</v>
       </c>
       <c r="W39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X39" t="n">
         <v>0</v>
@@ -3753,7 +3753,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Di Gennaro</t>
+          <t>Gollini</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -3781,7 +3781,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>40.7</v>
+        <v>39.1</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -3789,22 +3789,22 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M40" t="n">
         <v>3</v>
       </c>
       <c r="N40" t="n">
-        <v>2.56</v>
+        <v>-4.37</v>
       </c>
       <c r="O40" t="n">
-        <v>0.018</v>
+        <v>0.123</v>
       </c>
       <c r="P40" t="n">
         <v>0</v>
@@ -3828,7 +3828,7 @@
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X40" t="n">
         <v>0</v>
@@ -3840,7 +3840,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Gollini</t>
+          <t>Lezzerini</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>40</v>
+        <v>30.8</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -3885,13 +3885,11 @@
         <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>3</v>
-      </c>
-      <c r="N41" t="n">
-        <v>-4.37</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="n">
-        <v>0.123</v>
+        <v>0</v>
       </c>
       <c r="P41" t="n">
         <v>0</v>
@@ -3927,7 +3925,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Sommariva</t>
+          <t>Stolz</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3955,7 +3953,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>31.4</v>
+        <v>30.8</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -3963,22 +3961,22 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>5.75</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="M42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N42" t="n">
         <v>0</v>
       </c>
       <c r="O42" t="n">
-        <v>0.026</v>
+        <v>0</v>
       </c>
       <c r="P42" t="n">
         <v>0</v>
@@ -4002,7 +4000,7 @@
         <v>0</v>
       </c>
       <c r="W42" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X42" t="n">
         <v>0</v>
@@ -4014,7 +4012,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lezzerini</t>
+          <t>Torriani</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4024,7 +4022,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -4042,7 +4040,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -4059,9 +4057,11 @@
         <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>1</v>
-      </c>
-      <c r="N43" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0</v>
+      </c>
       <c r="O43" t="n">
         <v>0</v>
       </c>
@@ -4099,7 +4099,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Stolz</t>
+          <t>De Marzi</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -4127,7 +4127,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -4144,11 +4144,9 @@
         <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>2</v>
-      </c>
-      <c r="N44" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" t="n">
         <v>0</v>
       </c>
@@ -4186,7 +4184,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Torriani</t>
+          <t>Russo A.</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -4196,7 +4194,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -4214,7 +4212,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -4231,11 +4229,9 @@
         <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>2</v>
-      </c>
-      <c r="N45" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="n">
         <v>0</v>
       </c>
@@ -4273,7 +4269,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>De Marzi</t>
+          <t>Siviero</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4283,7 +4279,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -4301,7 +4297,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -4358,7 +4354,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Russo A.</t>
+          <t>Sommariva</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4368,7 +4364,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -4386,7 +4382,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>31.3</v>
+        <v>30.5</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -4394,20 +4390,22 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="M47" t="n">
-        <v>1</v>
-      </c>
-      <c r="N47" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0</v>
+      </c>
       <c r="O47" t="n">
-        <v>0</v>
+        <v>0.026</v>
       </c>
       <c r="P47" t="n">
         <v>0</v>
@@ -4431,7 +4429,7 @@
         <v>0</v>
       </c>
       <c r="W47" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X47" t="n">
         <v>0</v>
@@ -4443,7 +4441,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Siviero</t>
+          <t>Desplanches</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -4453,7 +4451,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -4470,39 +4468,19 @@
           <t>3a Fascia</t>
         </is>
       </c>
-      <c r="H48" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J48" t="n">
-        <v>0</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
-      </c>
-      <c r="L48" t="n">
-        <v>0</v>
-      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
       <c r="M48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N48" t="inlineStr"/>
-      <c r="O48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>0</v>
-      </c>
-      <c r="R48" t="n">
-        <v>0</v>
-      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
       <c r="S48" t="n">
         <v>0</v>
       </c>
@@ -4515,12 +4493,8 @@
       <c r="V48" t="n">
         <v>0</v>
       </c>
-      <c r="W48" t="n">
-        <v>0</v>
-      </c>
-      <c r="X48" t="n">
-        <v>0</v>
-      </c>
+      <c r="W48" t="inlineStr"/>
+      <c r="X48" t="inlineStr"/>
       <c r="Y48" t="inlineStr"/>
       <c r="Z48" t="inlineStr"/>
       <c r="AA48" t="inlineStr"/>
@@ -4528,7 +4502,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Desplanches</t>
+          <t>Lolic</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -4589,7 +4563,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Lolic</t>
+          <t>Renzetti</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4599,7 +4573,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -4650,7 +4624,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Renzetti</t>
+          <t>Strajnar</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4660,7 +4634,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -4711,7 +4685,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Strajnar</t>
+          <t>Montipò</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4721,7 +4695,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -4733,24 +4707,46 @@
       <c r="F52" t="n">
         <v>1</v>
       </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>3a Fascia</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Low Cost</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Affare</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>35</v>
+      </c>
+      <c r="K52" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="L52" t="n">
+        <v>4.94</v>
+      </c>
       <c r="M52" t="n">
-        <v>0</v>
-      </c>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="P52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>1</v>
+      </c>
+      <c r="R52" t="n">
+        <v>0</v>
+      </c>
       <c r="S52" t="n">
         <v>0</v>
       </c>
@@ -4763,8 +4759,12 @@
       <c r="V52" t="n">
         <v>0</v>
       </c>
-      <c r="W52" t="inlineStr"/>
-      <c r="X52" t="inlineStr"/>
+      <c r="W52" t="n">
+        <v>54</v>
+      </c>
+      <c r="X52" t="n">
+        <v>3</v>
+      </c>
       <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr"/>
       <c r="AA52" t="inlineStr"/>
@@ -4772,7 +4772,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Montipò</t>
+          <t>Padelli</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -4800,7 +4800,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>62.8</v>
+        <v>47.6</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -4808,28 +4808,28 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="K53" t="n">
-        <v>6.2</v>
+        <v>6.25</v>
       </c>
       <c r="L53" t="n">
-        <v>4.94</v>
+        <v>5.25</v>
       </c>
       <c r="M53" t="n">
         <v>3</v>
       </c>
       <c r="N53" t="n">
-        <v>0.29</v>
+        <v>1.19</v>
       </c>
       <c r="O53" t="n">
-        <v>0.947</v>
+        <v>0.026</v>
       </c>
       <c r="P53" t="n">
         <v>0</v>
       </c>
       <c r="Q53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R53" t="n">
         <v>0</v>
@@ -4847,10 +4847,10 @@
         <v>0</v>
       </c>
       <c r="W53" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="X53" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr"/>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>33.4</v>
+        <v>32.6</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -4946,7 +4946,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Piana</t>
+          <t>Grandi</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -4974,7 +4974,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -4991,11 +4991,9 @@
         <v>0</v>
       </c>
       <c r="M55" t="n">
-        <v>2</v>
-      </c>
-      <c r="N55" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N55" t="inlineStr"/>
       <c r="O55" t="n">
         <v>0</v>
       </c>
@@ -5033,7 +5031,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Grandi</t>
+          <t>Satalino</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5043,7 +5041,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -5061,7 +5059,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -5118,7 +5116,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Satalino</t>
+          <t>Bleve</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -5128,7 +5126,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -5146,7 +5144,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>31.3</v>
+        <v>30.8</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -5203,7 +5201,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Bleve</t>
+          <t>Pozzi</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -5213,7 +5211,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -5230,39 +5228,19 @@
           <t>Low Cost</t>
         </is>
       </c>
-      <c r="H58" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J58" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" t="n">
-        <v>0</v>
-      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N58" t="inlineStr"/>
-      <c r="O58" t="n">
-        <v>0</v>
-      </c>
-      <c r="P58" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q58" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" t="n">
-        <v>0</v>
-      </c>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
       <c r="S58" t="n">
         <v>0</v>
       </c>
@@ -5275,12 +5253,8 @@
       <c r="V58" t="n">
         <v>0</v>
       </c>
-      <c r="W58" t="n">
-        <v>0</v>
-      </c>
-      <c r="X58" t="n">
-        <v>0</v>
-      </c>
+      <c r="W58" t="inlineStr"/>
+      <c r="X58" t="inlineStr"/>
       <c r="Y58" t="inlineStr"/>
       <c r="Z58" t="inlineStr"/>
       <c r="AA58" t="inlineStr"/>
@@ -5288,7 +5262,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Pozzi</t>
+          <t>Penev</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -5298,7 +5272,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -5349,7 +5323,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Penev</t>
+          <t>Pisseri</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5359,7 +5333,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -5410,7 +5384,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Pisseri</t>
+          <t>Grabara</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5420,7 +5394,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -5471,7 +5445,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Grabara</t>
+          <t>Mrozek</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5481,7 +5455,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -5493,9 +5467,9 @@
       <c r="F62" t="n">
         <v>1</v>
       </c>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>Low Cost</t>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>Scommessa</t>
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
@@ -5532,7 +5506,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mrozek</t>
+          <t>Ghidotti</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5542,7 +5516,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -5593,7 +5567,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ghidotti</t>
+          <t>Pompei</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5603,7 +5577,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -5651,69 +5625,8 @@
       <c r="Z64" t="inlineStr"/>
       <c r="AA64" t="inlineStr"/>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Pompei</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Por</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Atalanta</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" t="n">
-        <v>1</v>
-      </c>
-      <c r="F65" t="n">
-        <v>1</v>
-      </c>
-      <c r="G65" s="7" t="inlineStr">
-        <is>
-          <t>Scommessa</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="n">
-        <v>0</v>
-      </c>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr"/>
-      <c r="S65" t="n">
-        <v>0</v>
-      </c>
-      <c r="T65" t="n">
-        <v>0</v>
-      </c>
-      <c r="U65" t="n">
-        <v>0</v>
-      </c>
-      <c r="V65" t="n">
-        <v>0</v>
-      </c>
-      <c r="W65" t="inlineStr"/>
-      <c r="X65" t="inlineStr"/>
-      <c r="Y65" t="inlineStr"/>
-      <c r="Z65" t="inlineStr"/>
-      <c r="AA65" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AA65"/>
+  <autoFilter ref="A1:AA64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -39665,7 +39578,7 @@
         <v>3</v>
       </c>
       <c r="T31" t="n">
-        <v>6.67</v>
+        <v>6.83</v>
       </c>
       <c r="U31" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-09-11
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Portieri'!$A$1:$AA$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Difensori'!$A$1:$AA$191</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Centrocampisti'!$A$1:$AA$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Centrocampisti'!$A$1:$AA$194</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Attaccanti'!$A$1:$AA$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21090,7 +21090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA193"/>
+  <dimension ref="A1:AA194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -35482,27 +35482,27 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Aboukhlal</t>
+          <t>Forson O.</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>W;A</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E174" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F174" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G174" s="6" t="inlineStr">
         <is>
@@ -35510,7 +35510,7 @@
         </is>
       </c>
       <c r="H174" t="n">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="I174" t="inlineStr">
         <is>
@@ -35518,20 +35518,20 @@
         </is>
       </c>
       <c r="J174" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K174" t="n">
-        <v>5.77</v>
+        <v>5.67</v>
       </c>
       <c r="L174" t="n">
-        <v>5.64</v>
+        <v>5.67</v>
       </c>
       <c r="M174" t="n">
         <v>1</v>
       </c>
       <c r="N174" t="inlineStr"/>
       <c r="O174" t="n">
-        <v>0.289</v>
+        <v>0.158</v>
       </c>
       <c r="P174" t="n">
         <v>0</v>
@@ -35546,7 +35546,7 @@
         <v>2</v>
       </c>
       <c r="T174" t="n">
-        <v>5.5</v>
+        <v>5.75</v>
       </c>
       <c r="U174" t="n">
         <v>0</v>
@@ -35555,7 +35555,7 @@
         <v>0</v>
       </c>
       <c r="W174" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X174" t="n">
         <v>0</v>
@@ -35567,21 +35567,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Hasa</t>
+          <t>Aboukhlal</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>C;T</t>
+          <t>W;A</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E175" t="n">
         <v>5</v>
@@ -35595,7 +35595,7 @@
         </is>
       </c>
       <c r="H175" t="n">
-        <v>6.4</v>
+        <v>8.5</v>
       </c>
       <c r="I175" t="inlineStr">
         <is>
@@ -35603,20 +35603,20 @@
         </is>
       </c>
       <c r="J175" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K175" t="n">
-        <v>0</v>
+        <v>5.77</v>
       </c>
       <c r="L175" t="n">
-        <v>0</v>
+        <v>5.64</v>
       </c>
       <c r="M175" t="n">
         <v>1</v>
       </c>
       <c r="N175" t="inlineStr"/>
       <c r="O175" t="n">
-        <v>0</v>
+        <v>0.289</v>
       </c>
       <c r="P175" t="n">
         <v>0</v>
@@ -35628,10 +35628,10 @@
         <v>0</v>
       </c>
       <c r="S175" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T175" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="U175" t="n">
         <v>0</v>
@@ -35640,7 +35640,7 @@
         <v>0</v>
       </c>
       <c r="W175" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X175" t="n">
         <v>0</v>
@@ -35652,21 +35652,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Przyborek</t>
+          <t>Hasa</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>W;T</t>
+          <t>C;T</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E176" t="n">
         <v>5</v>
@@ -35713,10 +35713,10 @@
         <v>0</v>
       </c>
       <c r="S176" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T176" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U176" t="n">
         <v>0</v>
@@ -35737,46 +35737,66 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Grillitsch</t>
+          <t>Przyborek</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>M;C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E177" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F177" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G177" s="6" t="inlineStr">
         <is>
           <t>Low Cost</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr"/>
-      <c r="J177" t="inlineStr"/>
-      <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
+      <c r="H177" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J177" t="n">
+        <v>0</v>
+      </c>
+      <c r="K177" t="n">
+        <v>0</v>
+      </c>
+      <c r="L177" t="n">
+        <v>0</v>
+      </c>
       <c r="M177" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr"/>
-      <c r="P177" t="inlineStr"/>
-      <c r="Q177" t="inlineStr"/>
-      <c r="R177" t="inlineStr"/>
+      <c r="O177" t="n">
+        <v>0</v>
+      </c>
+      <c r="P177" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>0</v>
+      </c>
+      <c r="R177" t="n">
+        <v>0</v>
+      </c>
       <c r="S177" t="n">
         <v>0</v>
       </c>
@@ -35789,8 +35809,12 @@
       <c r="V177" t="n">
         <v>0</v>
       </c>
-      <c r="W177" t="inlineStr"/>
-      <c r="X177" t="inlineStr"/>
+      <c r="W177" t="n">
+        <v>0</v>
+      </c>
+      <c r="X177" t="n">
+        <v>0</v>
+      </c>
       <c r="Y177" t="inlineStr"/>
       <c r="Z177" t="inlineStr"/>
       <c r="AA177" t="inlineStr"/>
@@ -35798,27 +35822,27 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Fernandez T.</t>
+          <t>Grillitsch</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>T;A</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D178" t="n">
         <v>4</v>
       </c>
       <c r="E178" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F178" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G178" s="6" t="inlineStr">
         <is>
@@ -35839,10 +35863,10 @@
       <c r="Q178" t="inlineStr"/>
       <c r="R178" t="inlineStr"/>
       <c r="S178" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T178" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U178" t="n">
         <v>0</v>
@@ -35859,24 +35883,24 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Stankovic A.</t>
+          <t>Fernandez T.</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>M;C</t>
+          <t>T;A</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E179" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F179" t="n">
         <v>4</v>
@@ -35900,10 +35924,10 @@
       <c r="Q179" t="inlineStr"/>
       <c r="R179" t="inlineStr"/>
       <c r="S179" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T179" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U179" t="n">
         <v>0</v>
@@ -35920,7 +35944,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Colombo L.</t>
+          <t>Stankovic A.</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -35930,17 +35954,17 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="D180" t="n">
         <v>2</v>
       </c>
       <c r="E180" t="n">
+        <v>7</v>
+      </c>
+      <c r="F180" t="n">
         <v>4</v>
-      </c>
-      <c r="F180" t="n">
-        <v>2</v>
       </c>
       <c r="G180" s="6" t="inlineStr">
         <is>
@@ -35961,10 +35985,10 @@
       <c r="Q180" t="inlineStr"/>
       <c r="R180" t="inlineStr"/>
       <c r="S180" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T180" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U180" t="n">
         <v>0</v>
@@ -35981,12 +36005,12 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Foe Ondoa</t>
+          <t>Colombo L.</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -35998,10 +36022,10 @@
         <v>2</v>
       </c>
       <c r="E181" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F181" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G181" s="6" t="inlineStr">
         <is>
@@ -36025,7 +36049,7 @@
         <v>1</v>
       </c>
       <c r="T181" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="U181" t="n">
         <v>0</v>
@@ -36042,27 +36066,27 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Jovanovic</t>
+          <t>Foe Ondoa</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>W;T</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D182" t="n">
         <v>2</v>
       </c>
       <c r="E182" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G182" s="6" t="inlineStr">
         <is>
@@ -36083,10 +36107,10 @@
       <c r="Q182" t="inlineStr"/>
       <c r="R182" t="inlineStr"/>
       <c r="S182" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T182" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U182" t="n">
         <v>0</v>
@@ -36103,7 +36127,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Chakvetadze</t>
+          <t>Jovanovic</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -36117,13 +36141,13 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E183" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F183" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G183" s="6" t="inlineStr">
         <is>
@@ -36164,66 +36188,46 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Liteta</t>
+          <t>Chakvetadze</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>M;C</t>
+          <t>W;T</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="D184" t="n">
         <v>1</v>
       </c>
       <c r="E184" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F184" t="n">
-        <v>1</v>
-      </c>
-      <c r="G184" s="7" t="inlineStr">
-        <is>
-          <t>Scommessa</t>
-        </is>
-      </c>
-      <c r="H184" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J184" t="n">
-        <v>4</v>
-      </c>
-      <c r="K184" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="L184" t="n">
-        <v>5.75</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G184" s="6" t="inlineStr">
+        <is>
+          <t>Low Cost</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
       <c r="M184" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N184" t="inlineStr"/>
-      <c r="O184" t="n">
-        <v>0.105</v>
-      </c>
-      <c r="P184" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q184" t="n">
-        <v>0</v>
-      </c>
-      <c r="R184" t="n">
-        <v>0</v>
-      </c>
+      <c r="O184" t="inlineStr"/>
+      <c r="P184" t="inlineStr"/>
+      <c r="Q184" t="inlineStr"/>
+      <c r="R184" t="inlineStr"/>
       <c r="S184" t="n">
         <v>0</v>
       </c>
@@ -36236,12 +36240,8 @@
       <c r="V184" t="n">
         <v>0</v>
       </c>
-      <c r="W184" t="n">
-        <v>0</v>
-      </c>
-      <c r="X184" t="n">
-        <v>0</v>
-      </c>
+      <c r="W184" t="inlineStr"/>
+      <c r="X184" t="inlineStr"/>
       <c r="Y184" t="inlineStr"/>
       <c r="Z184" t="inlineStr"/>
       <c r="AA184" t="inlineStr"/>
@@ -36249,21 +36249,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Forson O.</t>
+          <t>Liteta</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>W;T</t>
+          <t>M;C</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E185" t="n">
         <v>1</v>
@@ -36277,7 +36277,7 @@
         </is>
       </c>
       <c r="H185" t="n">
-        <v>10</v>
+        <v>10.7</v>
       </c>
       <c r="I185" t="inlineStr">
         <is>
@@ -36285,20 +36285,20 @@
         </is>
       </c>
       <c r="J185" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K185" t="n">
-        <v>5.67</v>
+        <v>5.75</v>
       </c>
       <c r="L185" t="n">
-        <v>5.67</v>
+        <v>5.75</v>
       </c>
       <c r="M185" t="n">
         <v>1</v>
       </c>
       <c r="N185" t="inlineStr"/>
       <c r="O185" t="n">
-        <v>0.158</v>
+        <v>0.105</v>
       </c>
       <c r="P185" t="n">
         <v>0</v>
@@ -36310,10 +36310,10 @@
         <v>0</v>
       </c>
       <c r="S185" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T185" t="n">
-        <v>5.75</v>
+        <v>0</v>
       </c>
       <c r="U185" t="n">
         <v>0</v>
@@ -36867,8 +36867,69 @@
       <c r="Z193" t="inlineStr"/>
       <c r="AA193" t="inlineStr"/>
     </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Libra</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>C;T</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>1</v>
+      </c>
+      <c r="E194" t="n">
+        <v>1</v>
+      </c>
+      <c r="F194" t="n">
+        <v>1</v>
+      </c>
+      <c r="G194" s="7" t="inlineStr">
+        <is>
+          <t>Scommessa</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr"/>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="inlineStr"/>
+      <c r="M194" t="n">
+        <v>0</v>
+      </c>
+      <c r="N194" t="inlineStr"/>
+      <c r="O194" t="inlineStr"/>
+      <c r="P194" t="inlineStr"/>
+      <c r="Q194" t="inlineStr"/>
+      <c r="R194" t="inlineStr"/>
+      <c r="S194" t="n">
+        <v>0</v>
+      </c>
+      <c r="T194" t="n">
+        <v>0</v>
+      </c>
+      <c r="U194" t="n">
+        <v>0</v>
+      </c>
+      <c r="V194" t="n">
+        <v>0</v>
+      </c>
+      <c r="W194" t="inlineStr"/>
+      <c r="X194" t="inlineStr"/>
+      <c r="Y194" t="inlineStr"/>
+      <c r="Z194" t="inlineStr"/>
+      <c r="AA194" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA193"/>
+  <autoFilter ref="A1:AA194"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-09-12
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -1200,10 +1200,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T8" t="n">
-        <v>2.5</v>
+        <v>2.88</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -2190,10 +2190,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T20" t="n">
-        <v>3.67</v>
+        <v>3.25</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -9149,10 +9149,10 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T41" t="n">
-        <v>4.67</v>
+        <v>5.12</v>
       </c>
       <c r="U41" t="n">
         <v>0</v>
@@ -11571,16 +11571,16 @@
         <v>0</v>
       </c>
       <c r="S69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T69" t="n">
-        <v>4.75</v>
+        <v>5.67</v>
       </c>
       <c r="U69" t="n">
         <v>0</v>
       </c>
       <c r="V69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W69" t="n">
         <v>1</v>
@@ -13287,13 +13287,13 @@
         <v>0</v>
       </c>
       <c r="S93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T93" t="n">
-        <v>6.33</v>
+        <v>7.12</v>
       </c>
       <c r="U93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V93" t="n">
         <v>1</v>
@@ -13894,10 +13894,10 @@
         <v>0</v>
       </c>
       <c r="S100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T100" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="U100" t="n">
         <v>0</v>
@@ -14068,16 +14068,16 @@
         <v>0</v>
       </c>
       <c r="S102" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T102" t="n">
-        <v>5.67</v>
+        <v>5.62</v>
       </c>
       <c r="U102" t="n">
         <v>0</v>
       </c>
       <c r="V102" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W102" t="n">
         <v>3</v>
@@ -16053,10 +16053,10 @@
         <v>0</v>
       </c>
       <c r="S125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T125" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U125" t="n">
         <v>0</v>
@@ -16223,7 +16223,7 @@
         <v>0</v>
       </c>
       <c r="S127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T127" t="n">
         <v>5</v>
@@ -16874,10 +16874,10 @@
       <c r="Q136" t="inlineStr"/>
       <c r="R136" t="inlineStr"/>
       <c r="S136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T136" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U136" t="n">
         <v>0</v>
@@ -16935,10 +16935,10 @@
       <c r="Q137" t="inlineStr"/>
       <c r="R137" t="inlineStr"/>
       <c r="S137" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T137" t="n">
-        <v>6.25</v>
+        <v>6.17</v>
       </c>
       <c r="U137" t="n">
         <v>0</v>
@@ -19112,7 +19112,7 @@
         <v>0</v>
       </c>
       <c r="S164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T164" t="n">
         <v>5</v>
@@ -19626,10 +19626,10 @@
         <v>0</v>
       </c>
       <c r="S170" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T170" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="U170" t="n">
         <v>1</v>
@@ -23318,10 +23318,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T25" t="n">
-        <v>5</v>
+        <v>5.38</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -24293,13 +24293,13 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T38" t="n">
-        <v>5.33</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="U38" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V38" t="n">
         <v>0</v>
@@ -26602,16 +26602,16 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T65" t="n">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
       </c>
       <c r="V65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W65" t="n">
         <v>5</v>
@@ -27557,10 +27557,10 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T76" t="n">
-        <v>5.17</v>
+        <v>5.5</v>
       </c>
       <c r="U76" t="n">
         <v>0</v>
@@ -27731,10 +27731,10 @@
         <v>0</v>
       </c>
       <c r="S78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T78" t="n">
-        <v>6.25</v>
+        <v>6.17</v>
       </c>
       <c r="U78" t="n">
         <v>0</v>
@@ -30125,16 +30125,16 @@
         <v>0</v>
       </c>
       <c r="S108" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T108" t="n">
-        <v>6.17</v>
+        <v>6.5</v>
       </c>
       <c r="U108" t="n">
         <v>0</v>
       </c>
       <c r="V108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W108" t="n">
         <v>4</v>
@@ -30297,10 +30297,10 @@
         <v>0</v>
       </c>
       <c r="S110" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T110" t="n">
-        <v>5.67</v>
+        <v>5.75</v>
       </c>
       <c r="U110" t="n">
         <v>0</v>
@@ -30817,10 +30817,10 @@
         <v>0</v>
       </c>
       <c r="S116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T116" t="n">
-        <v>5.5</v>
+        <v>5.17</v>
       </c>
       <c r="U116" t="n">
         <v>0</v>
@@ -33726,10 +33726,10 @@
         <v>0</v>
       </c>
       <c r="S153" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T153" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U153" t="n">
         <v>0</v>
@@ -39290,13 +39290,13 @@
         <v>1</v>
       </c>
       <c r="S27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T27" t="n">
-        <v>6.17</v>
+        <v>7.12</v>
       </c>
       <c r="U27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V27" t="n">
         <v>0</v>
@@ -39893,10 +39893,10 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T34" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="U34" t="n">
         <v>1</v>
@@ -40065,10 +40065,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T36" t="n">
-        <v>5.5</v>
+        <v>5.75</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -40278,13 +40278,13 @@
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T39" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="U39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V39" t="n">
         <v>0</v>
@@ -42344,10 +42344,10 @@
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T65" t="n">
-        <v>5.5</v>
+        <v>5.75</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>

</xml_diff>